<commit_message>
Zwischenergebnisse: neue finale Ergebnisse nach vollständiger Korrektur
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Korrektur.xlsx
+++ b/src/evaluation/data/Korrektur.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99EB11FF-E984-468F-A1D3-80A2DB7B3F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA932D75-9979-4F20-B3BF-E6C66ED7BE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="naive_max size" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="66">
   <si>
     <t>faithfulness</t>
   </si>
@@ -237,6 +237,12 @@
   </si>
   <si>
     <t>Reranking</t>
+  </si>
+  <si>
+    <t>Differenz zu 500</t>
+  </si>
+  <si>
+    <t>Total Tokens</t>
   </si>
 </sst>
 </file>
@@ -2698,29 +2704,35 @@
       <c r="B39">
         <v>0.78230560730060283</v>
       </c>
+      <c r="C39">
+        <v>0.77333463461025653</v>
+      </c>
+      <c r="D39">
+        <v>0.76581336053452265</v>
+      </c>
       <c r="E39">
         <f>AVERAGE(B39:D39)</f>
-        <v>0.78230560730060283</v>
+        <v>0.77381786748179404</v>
       </c>
       <c r="G39">
         <f>E39-E3</f>
-        <v>-2.9463421288425273E-2</v>
+        <v>-3.7951161107234066E-2</v>
       </c>
       <c r="H39">
         <f>G39*100</f>
-        <v>-2.9463421288425273</v>
+        <v>-3.7951161107234066</v>
       </c>
       <c r="I39">
         <f>G39/E3*100</f>
-        <v>-3.6295325703219987</v>
+        <v>-4.6751181396016879</v>
       </c>
       <c r="K39">
         <f>E39-E21</f>
-        <v>-2.8292633445053506E-2</v>
+        <v>-3.6780373263862298E-2</v>
       </c>
       <c r="L39">
         <f>K39*100</f>
-        <v>-2.8292633445053506</v>
+        <v>-3.6780373263862298</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -2730,29 +2742,35 @@
       <c r="B40">
         <v>0.70662972085385878</v>
       </c>
+      <c r="C40">
+        <v>0.70950328407224961</v>
+      </c>
+      <c r="D40">
+        <v>0.71568144499178987</v>
+      </c>
       <c r="E40">
         <f t="shared" ref="E40:E53" si="4">AVERAGE(B40:D40)</f>
-        <v>0.70662972085385878</v>
+        <v>0.71060481663929931</v>
       </c>
       <c r="G40">
         <f t="shared" ref="G40:G53" si="5">E40-E22</f>
-        <v>-6.2260536398467403E-3</v>
+        <v>-2.2509578544062103E-3</v>
       </c>
       <c r="H40">
         <f t="shared" ref="H40:H53" si="6">G40*100</f>
-        <v>-0.62260536398467403</v>
+        <v>-0.22509578544062103</v>
       </c>
       <c r="I40">
         <f t="shared" ref="I40:I53" si="7">G40/E22*100</f>
-        <v>-0.87339597470030961</v>
+        <v>-0.31576623700704637</v>
       </c>
       <c r="K40">
         <f t="shared" ref="K40:K53" si="8">E40-E22</f>
-        <v>-6.2260536398467403E-3</v>
+        <v>-2.2509578544062103E-3</v>
       </c>
       <c r="L40">
         <f t="shared" ref="L40:L53" si="9">K40*100</f>
-        <v>-0.62260536398467403</v>
+        <v>-0.22509578544062103</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -2762,29 +2780,35 @@
       <c r="B41">
         <v>0.64233716472058711</v>
       </c>
+      <c r="C41">
+        <v>0.63414750954912147</v>
+      </c>
+      <c r="D41">
+        <v>0.63594348655962396</v>
+      </c>
       <c r="E41">
         <f t="shared" si="4"/>
-        <v>0.64233716472058711</v>
+        <v>0.63747605360977744</v>
       </c>
       <c r="G41">
         <f t="shared" si="5"/>
-        <v>-3.9910600273078689E-3</v>
+        <v>-8.8521711381175372E-3</v>
       </c>
       <c r="H41">
         <f t="shared" si="6"/>
-        <v>-0.39910600273078689</v>
+        <v>-0.88521711381175372</v>
       </c>
       <c r="I41">
         <f t="shared" si="7"/>
-        <v>-0.61749740681131648</v>
+        <v>-1.369609247928232</v>
       </c>
       <c r="K41">
         <f t="shared" si="8"/>
-        <v>-3.9910600273078689E-3</v>
+        <v>-8.8521711381175372E-3</v>
       </c>
       <c r="L41">
         <f t="shared" si="9"/>
-        <v>-0.39910600273078689</v>
+        <v>-0.88521711381175372</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
@@ -2794,6 +2818,12 @@
       <c r="B42">
         <v>0.77033469535003851</v>
       </c>
+      <c r="C42">
+        <v>0.77033469535003851</v>
+      </c>
+      <c r="D42">
+        <v>0.77033469535003851</v>
+      </c>
       <c r="E42">
         <f t="shared" si="4"/>
         <v>0.77033469535003851</v>
@@ -2826,29 +2856,35 @@
       <c r="B43">
         <v>0.27229885477857502</v>
       </c>
+      <c r="C43">
+        <v>0.28870595463342408</v>
+      </c>
+      <c r="D43">
+        <v>0.27529461421695628</v>
+      </c>
       <c r="E43">
         <f t="shared" si="4"/>
-        <v>0.27229885477857502</v>
+        <v>0.27876647454298514</v>
       </c>
       <c r="G43">
         <f t="shared" si="5"/>
-        <v>-6.9997475486751615E-3</v>
+        <v>-5.3212778426503515E-4</v>
       </c>
       <c r="H43">
         <f t="shared" si="6"/>
-        <v>-0.69997475486751615</v>
+        <v>-5.3212778426503515E-2</v>
       </c>
       <c r="I43">
         <f t="shared" si="7"/>
-        <v>-2.5061878184673683</v>
+        <v>-0.19052289550720652</v>
       </c>
       <c r="K43">
         <f t="shared" si="8"/>
-        <v>-6.9997475486751615E-3</v>
+        <v>-5.3212778426503515E-4</v>
       </c>
       <c r="L43">
         <f t="shared" si="9"/>
-        <v>-0.69997475486751615</v>
+        <v>-5.3212778426503515E-2</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -2858,29 +2894,35 @@
       <c r="B44">
         <v>0.74357374507422869</v>
       </c>
+      <c r="C44">
+        <v>0.74676142622550323</v>
+      </c>
+      <c r="D44">
+        <v>0.73737061995840936</v>
+      </c>
       <c r="E44">
         <f t="shared" si="4"/>
-        <v>0.74357374507422869</v>
+        <v>0.74256859708604706</v>
       </c>
       <c r="G44">
         <f t="shared" si="5"/>
-        <v>-2.7090726296102985E-2</v>
+        <v>-2.8095874284284617E-2</v>
       </c>
       <c r="H44">
         <f t="shared" si="6"/>
-        <v>-2.7090726296102985</v>
+        <v>-2.8095874284284617</v>
       </c>
       <c r="I44">
         <f t="shared" si="7"/>
-        <v>-3.5152426642858599</v>
+        <v>-3.6456688128267882</v>
       </c>
       <c r="K44">
         <f t="shared" si="8"/>
-        <v>-2.7090726296102985E-2</v>
+        <v>-2.8095874284284617E-2</v>
       </c>
       <c r="L44">
         <f t="shared" si="9"/>
-        <v>-2.7090726296102985</v>
+        <v>-2.8095874284284617</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -2890,6 +2932,12 @@
       <c r="B45">
         <v>0.2670670747756958</v>
       </c>
+      <c r="C45">
+        <v>0.2670670747756958</v>
+      </c>
+      <c r="D45">
+        <v>0.2670670747756958</v>
+      </c>
       <c r="E45">
         <f t="shared" si="4"/>
         <v>0.2670670747756958</v>
@@ -2922,6 +2970,12 @@
       <c r="B46">
         <v>0.18656368553638461</v>
       </c>
+      <c r="C46">
+        <v>0.18656368553638461</v>
+      </c>
+      <c r="D46">
+        <v>0.18656368553638461</v>
+      </c>
       <c r="E46">
         <f t="shared" si="4"/>
         <v>0.18656368553638461</v>
@@ -2954,6 +3008,12 @@
       <c r="B47">
         <v>0.35048586130142212</v>
       </c>
+      <c r="C47">
+        <v>0.35048586130142212</v>
+      </c>
+      <c r="D47">
+        <v>0.35048586130142212</v>
+      </c>
       <c r="E47">
         <f t="shared" si="4"/>
         <v>0.35048586130142212</v>
@@ -2986,6 +3046,12 @@
       <c r="B48">
         <v>0.37083333333333329</v>
       </c>
+      <c r="C48">
+        <v>0.37083333333333329</v>
+      </c>
+      <c r="D48">
+        <v>0.37083333333333329</v>
+      </c>
       <c r="E48">
         <f t="shared" si="4"/>
         <v>0.37083333333333329</v>
@@ -3018,6 +3084,12 @@
       <c r="B49">
         <v>0.53448275862068961</v>
       </c>
+      <c r="C49">
+        <v>0.53448275862068961</v>
+      </c>
+      <c r="D49">
+        <v>0.53448275862068961</v>
+      </c>
       <c r="E49">
         <f t="shared" si="4"/>
         <v>0.53448275862068961</v>
@@ -3050,29 +3122,35 @@
       <c r="B50">
         <v>15.38659848221417</v>
       </c>
+      <c r="C50">
+        <v>14.819913833305749</v>
+      </c>
+      <c r="D50">
+        <v>16.057225159529981</v>
+      </c>
       <c r="E50">
         <f t="shared" si="4"/>
-        <v>15.38659848221417</v>
+        <v>15.421245825016634</v>
       </c>
       <c r="G50">
         <f t="shared" si="5"/>
-        <v>4.3261256711240037E-3</v>
+        <v>3.8973468473587403E-2</v>
       </c>
       <c r="H50">
         <f t="shared" si="6"/>
-        <v>0.43261256711240037</v>
+        <v>3.8973468473587403</v>
       </c>
       <c r="I50">
         <f t="shared" si="7"/>
-        <v>2.8124100073444808E-2</v>
+        <v>0.25336613193569896</v>
       </c>
       <c r="K50">
         <f t="shared" si="8"/>
-        <v>4.3261256711240037E-3</v>
+        <v>3.8973468473587403E-2</v>
       </c>
       <c r="L50">
         <f t="shared" si="9"/>
-        <v>0.43261256711240037</v>
+        <v>3.8973468473587403</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -3082,29 +3160,35 @@
       <c r="B51">
         <v>3247.1724137931028</v>
       </c>
+      <c r="C51">
+        <v>3291.6982758620688</v>
+      </c>
+      <c r="D51">
+        <v>3252.655172413793</v>
+      </c>
       <c r="E51">
         <f t="shared" si="4"/>
-        <v>3247.1724137931028</v>
+        <v>3263.8419540229884</v>
       </c>
       <c r="G51">
         <f t="shared" si="5"/>
-        <v>-45.18965517241395</v>
+        <v>-28.52011494252838</v>
       </c>
       <c r="H51">
         <f t="shared" si="6"/>
-        <v>-4518.965517241395</v>
+        <v>-2852.011494252838</v>
       </c>
       <c r="I51">
         <f t="shared" si="7"/>
-        <v>-1.3725603146258107</v>
+        <v>-0.86625086625085557</v>
       </c>
       <c r="K51">
         <f t="shared" si="8"/>
-        <v>-45.18965517241395</v>
+        <v>-28.52011494252838</v>
       </c>
       <c r="L51">
         <f t="shared" si="9"/>
-        <v>-4518.965517241395</v>
+        <v>-2852.011494252838</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
@@ -3114,29 +3198,35 @@
       <c r="B52">
         <v>288.75862068965517</v>
       </c>
+      <c r="C52">
+        <v>291.84482758620692</v>
+      </c>
+      <c r="D52">
+        <v>288.30172413793099</v>
+      </c>
       <c r="E52">
         <f t="shared" si="4"/>
-        <v>288.75862068965517</v>
+        <v>289.63505747126436</v>
       </c>
       <c r="G52">
         <f t="shared" si="5"/>
-        <v>-4.7356321839081374</v>
+        <v>-3.8591954022989512</v>
       </c>
       <c r="H52">
         <f t="shared" si="6"/>
-        <v>-473.56321839081374</v>
+        <v>-385.91954022989512</v>
       </c>
       <c r="I52">
         <f t="shared" si="7"/>
-        <v>-1.613534894650301</v>
+        <v>-1.3149134487350538</v>
       </c>
       <c r="K52">
         <f t="shared" si="8"/>
-        <v>-4.7356321839081374</v>
+        <v>-3.8591954022989512</v>
       </c>
       <c r="L52">
         <f t="shared" si="9"/>
-        <v>-473.56321839081374</v>
+        <v>-385.91954022989512</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
@@ -3146,29 +3236,35 @@
       <c r="B53">
         <v>3535.9310344827591</v>
       </c>
+      <c r="C53">
+        <v>3583.5431034482758</v>
+      </c>
+      <c r="D53">
+        <v>3540.9568965517242</v>
+      </c>
       <c r="E53">
         <f t="shared" si="4"/>
-        <v>3535.9310344827591</v>
+        <v>3553.477011494253</v>
       </c>
       <c r="G53">
         <f t="shared" si="5"/>
-        <v>-49.925287356321405</v>
+        <v>-32.379310344827445</v>
       </c>
       <c r="H53">
         <f t="shared" si="6"/>
-        <v>-4992.5287356321405</v>
+        <v>-3237.9310344827445</v>
       </c>
       <c r="I53">
         <f t="shared" si="7"/>
-        <v>-1.392283540538406</v>
+        <v>-0.90297288677258125</v>
       </c>
       <c r="K53">
         <f t="shared" si="8"/>
-        <v>-49.925287356321405</v>
+        <v>-32.379310344827445</v>
       </c>
       <c r="L53">
         <f t="shared" si="9"/>
-        <v>-4992.5287356321405</v>
+        <v>-3237.9310344827445</v>
       </c>
     </row>
   </sheetData>
@@ -3212,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>0.72975999949645065</v>
+        <v>0.73584911932200248</v>
       </c>
       <c r="C3">
         <v>0.72116700820050561</v>
@@ -3222,7 +3318,7 @@
       </c>
       <c r="E3">
         <f>AVERAGE(B3:D3)</f>
-        <v>0.72503221418166441</v>
+        <v>0.7270619207901815</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -3230,7 +3326,7 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>0.63322463768115933</v>
+        <v>0.63638649425287364</v>
       </c>
       <c r="C4">
         <v>0.62830459770114933</v>
@@ -3240,7 +3336,7 @@
       </c>
       <c r="E4">
         <f t="shared" ref="E4:E17" si="0">AVERAGE(B4:D4)</f>
-        <v>0.6319561052806929</v>
+        <v>0.63301005747126438</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -3248,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <v>0.54548941796646877</v>
+        <v>0.56125478924927452</v>
       </c>
       <c r="C5">
         <v>0.55694444442082325</v>
@@ -3258,7 +3354,7 @@
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>0.55434848693497896</v>
+        <v>0.55960361069591424</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -3266,7 +3362,7 @@
         <v>3</v>
       </c>
       <c r="B6">
-        <v>0.77965471478153314</v>
+        <v>0.77965471478153325</v>
       </c>
       <c r="C6">
         <v>0.78090565145557822</v>
@@ -3284,7 +3380,7 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>0.2574353724792644</v>
+        <v>0.25902734613947342</v>
       </c>
       <c r="C7">
         <v>0.26536264152215822</v>
@@ -3294,7 +3390,7 @@
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>0.26149491936854591</v>
+        <v>0.26202557725528225</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -3302,7 +3398,7 @@
         <v>5</v>
       </c>
       <c r="B8">
-        <v>0.67293952504504861</v>
+        <v>0.66823012671184989</v>
       </c>
       <c r="C8">
         <v>0.67146515595114276</v>
@@ -3312,7 +3408,7 @@
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>0.68211287304986656</v>
+        <v>0.68054307360546684</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3320,7 +3416,7 @@
         <v>6</v>
       </c>
       <c r="B9">
-        <v>0.26693576574325562</v>
+        <v>0.26693576995026447</v>
       </c>
       <c r="C9">
         <v>0.26693576574325562</v>
@@ -3330,7 +3426,7 @@
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>0.26693576574325562</v>
+        <v>0.26693576714559192</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3338,7 +3434,7 @@
         <v>7</v>
       </c>
       <c r="B10">
-        <v>0.1888626962900162</v>
+        <v>0.18886269467124106</v>
       </c>
       <c r="C10">
         <v>0.1888626962900162</v>
@@ -3348,7 +3444,7 @@
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>0.1888626962900162</v>
+        <v>0.18886269575042447</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -3356,7 +3452,7 @@
         <v>8</v>
       </c>
       <c r="B11">
-        <v>0.34839504957199102</v>
+        <v>0.34839504110980135</v>
       </c>
       <c r="C11">
         <v>0.34839504957199102</v>
@@ -3366,7 +3462,7 @@
       </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>0.34839504957199102</v>
+        <v>0.34839504675126109</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3392,7 +3488,7 @@
         <v>10</v>
       </c>
       <c r="B13">
-        <v>0.47413793103448282</v>
+        <v>0.47413793103448276</v>
       </c>
       <c r="C13">
         <v>0.47413793103448282</v>
@@ -3410,7 +3506,7 @@
         <v>11</v>
       </c>
       <c r="B14">
-        <v>14.247814110640819</v>
+        <v>14.247814110640821</v>
       </c>
       <c r="C14">
         <v>14.45260334631492</v>
@@ -3446,7 +3542,7 @@
         <v>13</v>
       </c>
       <c r="B16">
-        <v>275.69827586206901</v>
+        <v>275.69827586206895</v>
       </c>
       <c r="C16">
         <v>275.69827586206901</v>
@@ -3550,15 +3646,15 @@
       </c>
       <c r="K21">
         <f>E21-E3</f>
-        <v>8.6736814407363694E-2</v>
+        <v>8.4707107798846604E-2</v>
       </c>
       <c r="L21">
         <f>K21*100</f>
-        <v>8.6736814407363703</v>
+        <v>8.4707107798846604</v>
       </c>
       <c r="M21">
         <f>K21/E3*100</f>
-        <v>11.963166975313303</v>
+        <v>11.650604353861041</v>
       </c>
       <c r="N21" t="s">
         <v>22</v>
@@ -3594,15 +3690,15 @@
       </c>
       <c r="K22">
         <f t="shared" ref="K22:K35" si="4">E22-E4</f>
-        <v>4.7087408676614095E-2</v>
+        <v>4.6033456486042623E-2</v>
       </c>
       <c r="L22">
         <f t="shared" ref="L22:L31" si="5">K22*100</f>
-        <v>4.70874086766141</v>
+        <v>4.6033456486042628</v>
       </c>
       <c r="M22">
         <f t="shared" ref="M22:M35" si="6">K22/E4*100</f>
-        <v>7.451056850807622</v>
+        <v>7.2721524630961056</v>
       </c>
       <c r="N22" t="s">
         <v>22</v>
@@ -3641,15 +3737,15 @@
       </c>
       <c r="K23">
         <f t="shared" si="4"/>
-        <v>9.5922905117474588E-2</v>
+        <v>9.0667781356539301E-2</v>
       </c>
       <c r="L23">
         <f t="shared" si="5"/>
-        <v>9.5922905117474588</v>
+        <v>9.0667781356539301</v>
       </c>
       <c r="M23">
         <f t="shared" si="6"/>
-        <v>17.30371911860664</v>
+        <v>16.20214373595379</v>
       </c>
       <c r="N23" t="s">
         <v>22</v>
@@ -3729,15 +3825,15 @@
       </c>
       <c r="K25">
         <f t="shared" si="4"/>
-        <v>1.5334818023067076E-2</v>
+        <v>1.4804160136330735E-2</v>
       </c>
       <c r="L25">
         <f t="shared" si="5"/>
-        <v>1.5334818023067076</v>
+        <v>1.4804160136330735</v>
       </c>
       <c r="M25">
         <f t="shared" si="6"/>
-        <v>5.8642890883300405</v>
+        <v>5.6498912401622396</v>
       </c>
       <c r="N25" t="s">
         <v>22</v>
@@ -3776,15 +3872,15 @@
       </c>
       <c r="K26">
         <f t="shared" si="4"/>
-        <v>7.8807225426481997E-2</v>
+        <v>8.0377024870881719E-2</v>
       </c>
       <c r="L26">
         <f t="shared" si="5"/>
-        <v>7.8807225426481997</v>
+        <v>8.0377024870881719</v>
       </c>
       <c r="M26">
         <f t="shared" si="6"/>
-        <v>11.553399523764847</v>
+        <v>11.810718231992311</v>
       </c>
       <c r="N26" t="s">
         <v>22</v>
@@ -3820,15 +3916,15 @@
       </c>
       <c r="K27">
         <f t="shared" si="4"/>
-        <v>1.494210958480835E-2</v>
+        <v>1.4942108182472047E-2</v>
       </c>
       <c r="L27">
         <f t="shared" si="5"/>
-        <v>1.494210958480835</v>
+        <v>1.4942108182472047</v>
       </c>
       <c r="M27">
         <f t="shared" si="6"/>
-        <v>5.5976423928069581</v>
+        <v>5.5976418380539963</v>
       </c>
       <c r="N27" t="s">
         <v>22</v>
@@ -3864,15 +3960,15 @@
       </c>
       <c r="K28">
         <f t="shared" si="4"/>
-        <v>1.5091622869173649E-2</v>
+        <v>1.5091623408765381E-2</v>
       </c>
       <c r="L28">
         <f t="shared" si="5"/>
-        <v>1.5091622869173649</v>
+        <v>1.509162340876538</v>
       </c>
       <c r="M28">
         <f t="shared" si="6"/>
-        <v>7.990790752028162</v>
+        <v>7.9907910605641463</v>
       </c>
       <c r="N28" t="s">
         <v>22</v>
@@ -3908,15 +4004,15 @@
       </c>
       <c r="K29">
         <f t="shared" si="4"/>
-        <v>1.3869841893513923E-2</v>
+        <v>1.3869844714243851E-2</v>
       </c>
       <c r="L29">
         <f t="shared" si="5"/>
-        <v>1.3869841893513923</v>
+        <v>1.3869844714243851</v>
       </c>
       <c r="M29">
         <f t="shared" si="6"/>
-        <v>3.9810674435682278</v>
+        <v>3.9810682854358479</v>
       </c>
       <c r="N29" t="s">
         <v>22</v>
@@ -7065,15 +7161,15 @@
       </c>
       <c r="K21">
         <f>E21-reranking!E21</f>
-        <v>4.1740975487461252E-2</v>
+        <v>2.8378779822343936E-2</v>
       </c>
       <c r="L21">
         <f>K21*100</f>
-        <v>4.1740975487461256</v>
+        <v>2.8378779822343936</v>
       </c>
       <c r="M21">
         <f>K21/reranking!E21*100</f>
-        <v>5.071095788887475</v>
+        <v>3.3926523026043389</v>
       </c>
       <c r="O21" t="s">
         <v>0</v>
@@ -7108,15 +7204,15 @@
       </c>
       <c r="Y21">
         <f>S21-reranking!E21</f>
-        <v>7.1760904024451899E-2</v>
+        <v>5.8398708359334583E-2</v>
       </c>
       <c r="Z21">
         <f>Y21*100</f>
-        <v>7.1760904024451904</v>
+        <v>5.8398708359334588</v>
       </c>
       <c r="AA21">
         <f>Y21/reranking!E21*100</f>
-        <v>8.7182058865507752</v>
+        <v>6.9815021514216591</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.25">
@@ -7150,15 +7246,15 @@
       </c>
       <c r="K22">
         <f>E22-reranking!E22</f>
-        <v>4.6707375478927116E-2</v>
+        <v>3.9379789272030674E-2</v>
       </c>
       <c r="L22">
         <f t="shared" ref="L22:L36" si="4">K22*100</f>
-        <v>4.6707375478927116</v>
+        <v>3.9379789272030674</v>
       </c>
       <c r="M22">
         <f>K22/reranking!E22*100</f>
-        <v>5.8541929287472119</v>
+        <v>4.8908517725434235</v>
       </c>
       <c r="O22" t="s">
         <v>1</v>
@@ -7193,15 +7289,15 @@
       </c>
       <c r="Y22">
         <f>S22-reranking!E22</f>
-        <v>3.8457854406130143E-2</v>
+        <v>3.1130268199233702E-2</v>
       </c>
       <c r="Z22">
         <f t="shared" ref="Z22:Z36" si="8">Y22*100</f>
-        <v>3.8457854406130143</v>
+        <v>3.1130268199233702</v>
       </c>
       <c r="AA22">
         <f>Y22/reranking!E22*100</f>
-        <v>4.8202172999579647</v>
+        <v>3.8662859862003311</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
@@ -7235,15 +7331,15 @@
       </c>
       <c r="K23">
         <f>E23-reranking!E23</f>
-        <v>7.0282567002842855E-3</v>
+        <v>-4.6296296659353864E-4</v>
       </c>
       <c r="L23">
         <f t="shared" si="4"/>
-        <v>0.70282567002842855</v>
+        <v>-4.6296296659353864E-2</v>
       </c>
       <c r="M23">
         <f>K23/reranking!E23*100</f>
-        <v>0.86262638083487997</v>
+        <v>-5.6304940231475059E-2</v>
       </c>
       <c r="O23" t="s">
         <v>2</v>
@@ -7278,15 +7374,15 @@
       </c>
       <c r="Y23">
         <f>S23-reranking!E23</f>
-        <v>2.7011494246256929E-2</v>
+        <v>1.9520274579379104E-2</v>
       </c>
       <c r="Z23">
         <f t="shared" si="8"/>
-        <v>2.7011494246256929</v>
+        <v>1.9520274579379104</v>
       </c>
       <c r="AA23">
         <f>Y23/reranking!E23*100</f>
-        <v>3.3153068415455436</v>
+        <v>2.3740298313296271</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
@@ -7320,15 +7416,15 @@
       </c>
       <c r="K24">
         <f>E24-reranking!E24</f>
-        <v>1.3770811963298102E-2</v>
+        <v>1.3856249311432367E-2</v>
       </c>
       <c r="L24">
         <f t="shared" si="4"/>
-        <v>1.3770811963298102</v>
+        <v>1.3856249311432367</v>
       </c>
       <c r="M24">
         <f>K24/reranking!E24*100</f>
-        <v>1.7456029721464348</v>
+        <v>1.7566233471129833</v>
       </c>
       <c r="O24" t="s">
         <v>3</v>
@@ -7360,15 +7456,15 @@
       </c>
       <c r="Y24">
         <f>S24-reranking!E24</f>
-        <v>9.8932850914809078E-3</v>
+        <v>9.978722439615173E-3</v>
       </c>
       <c r="Z24">
         <f t="shared" si="8"/>
-        <v>0.98932850914809078</v>
+        <v>0.9978722439615173</v>
       </c>
       <c r="AA24">
         <f>Y24/reranking!E24*100</f>
-        <v>1.2540834851284246</v>
+        <v>1.265050622128004</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.25">
@@ -7402,15 +7498,15 @@
       </c>
       <c r="K25">
         <f>E25-reranking!E25</f>
-        <v>3.3512788860404596E-2</v>
+        <v>3.5898160210962704E-2</v>
       </c>
       <c r="L25">
         <f t="shared" si="4"/>
-        <v>3.3512788860404594</v>
+        <v>3.5898160210962704</v>
       </c>
       <c r="M25">
         <f>K25/reranking!E25*100</f>
-        <v>10.075458986527359</v>
+        <v>10.870567748762102</v>
       </c>
       <c r="O25" t="s">
         <v>4</v>
@@ -7445,15 +7541,15 @@
       </c>
       <c r="Y25">
         <f>S25-reranking!E25</f>
-        <v>3.828273621247047E-2</v>
+        <v>4.0668107563028577E-2</v>
       </c>
       <c r="Z25">
         <f t="shared" si="8"/>
-        <v>3.828273621247047</v>
+        <v>4.0668107563028579</v>
       </c>
       <c r="AA25">
         <f>Y25/reranking!E25*100</f>
-        <v>11.50952074467655</v>
+        <v>12.314988174319891</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
@@ -7487,15 +7583,15 @@
       </c>
       <c r="K26">
         <f>E26-reranking!E26</f>
-        <v>6.0413411445845444E-2</v>
+        <v>5.410052242126806E-2</v>
       </c>
       <c r="L26">
         <f t="shared" si="4"/>
-        <v>6.0413411445845444</v>
+        <v>5.410052242126806</v>
       </c>
       <c r="M26">
         <f>K26/reranking!E26*100</f>
-        <v>8.3813226378124472</v>
+        <v>7.4403547830063612</v>
       </c>
       <c r="O26" t="s">
         <v>5</v>
@@ -7530,15 +7626,15 @@
       </c>
       <c r="Y26">
         <f>S26-reranking!E26</f>
-        <v>7.7813994984304191E-2</v>
+        <v>7.1501105959726807E-2</v>
       </c>
       <c r="Z26">
         <f t="shared" si="8"/>
-        <v>7.7813994984304191</v>
+        <v>7.1501105959726807</v>
       </c>
       <c r="AA26">
         <f>Y26/reranking!E26*100</f>
-        <v>10.795354575948595</v>
+        <v>9.8334280688675957</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.25">
@@ -7572,15 +7668,15 @@
       </c>
       <c r="K27">
         <f>E27-reranking!E27</f>
-        <v>2.8186261653900202E-2</v>
+        <v>2.8299510478973389E-2</v>
       </c>
       <c r="L27">
         <f t="shared" si="4"/>
-        <v>2.81862616539002</v>
+        <v>2.8299510478973389</v>
       </c>
       <c r="M27">
         <f>K27/reranking!E27*100</f>
-        <v>9.5696319647850725</v>
+        <v>9.6117772193023043</v>
       </c>
       <c r="O27" t="s">
         <v>6</v>
@@ -7615,15 +7711,15 @@
       </c>
       <c r="Y27">
         <f>S27-reranking!E27</f>
-        <v>2.3205141226450676E-2</v>
+        <v>2.3318390051523863E-2</v>
       </c>
       <c r="Z27">
         <f t="shared" si="8"/>
-        <v>2.3205141226450676</v>
+        <v>2.3318390051523865</v>
       </c>
       <c r="AA27">
         <f>Y27/reranking!E27*100</f>
-        <v>7.8784715743695184</v>
+        <v>7.9199663349149674</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.25">
@@ -7657,15 +7753,15 @@
       </c>
       <c r="K28">
         <f>E28-reranking!E28</f>
-        <v>4.3790395061175019E-2</v>
+        <v>4.4071515401204409E-2</v>
       </c>
       <c r="L28">
         <f t="shared" si="4"/>
-        <v>4.3790395061175023</v>
+        <v>4.4071515401204406</v>
       </c>
       <c r="M28">
         <f>K28/reranking!E28*100</f>
-        <v>20.833251511946969</v>
+        <v>20.995073730768098</v>
       </c>
       <c r="O28" t="s">
         <v>7</v>
@@ -7700,15 +7796,15 @@
       </c>
       <c r="Y28">
         <f>S28-reranking!E28</f>
-        <v>3.4909844398498535E-2</v>
+        <v>3.5190964738527925E-2</v>
       </c>
       <c r="Z28">
         <f t="shared" si="8"/>
-        <v>3.4909844398498535</v>
+        <v>3.5190964738527923</v>
       </c>
       <c r="AA28">
         <f>Y28/reranking!E28*100</f>
-        <v>16.608335402794101</v>
+        <v>16.764499532549834</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.25">
@@ -7742,15 +7838,15 @@
       </c>
       <c r="K29">
         <f>E29-reranking!E29</f>
-        <v>1.2347151835759462E-2</v>
+        <v>1.2292514244715336E-2</v>
       </c>
       <c r="L29">
         <f t="shared" si="4"/>
-        <v>1.2347151835759462</v>
+        <v>1.2292514244715336</v>
       </c>
       <c r="M29">
         <f>K29/reranking!E29*100</f>
-        <v>3.234470421161534</v>
+        <v>3.2196966789459833</v>
       </c>
       <c r="O29" t="s">
         <v>8</v>
@@ -7785,15 +7881,15 @@
       </c>
       <c r="Y29">
         <f>S29-reranking!E29</f>
-        <v>1.1348714431126894E-2</v>
+        <v>1.1294076840082767E-2</v>
       </c>
       <c r="Z29">
         <f t="shared" si="8"/>
-        <v>1.1348714431126894</v>
+        <v>1.1294076840082767</v>
       </c>
       <c r="AA29">
         <f>Y29/reranking!E29*100</f>
-        <v>2.9729189074502993</v>
+        <v>2.9581825955099652</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
@@ -7997,15 +8093,15 @@
       </c>
       <c r="K32">
         <f>E32-reranking!E32</f>
-        <v>-0.29857021775739057</v>
+        <v>1.2203696883957935</v>
       </c>
       <c r="L32">
         <f t="shared" si="4"/>
-        <v>-29.857021775739057</v>
+        <v>122.03696883957934</v>
       </c>
       <c r="M32">
         <f>K32/reranking!E32*100</f>
-        <v>-1.7606555630312881</v>
+        <v>7.9044809035613932</v>
       </c>
       <c r="O32" t="s">
         <v>11</v>
@@ -8037,15 +8133,15 @@
       </c>
       <c r="Y32">
         <f>S32-reranking!E32</f>
-        <v>4.9206207264428841</v>
+        <v>6.4395606325960681</v>
       </c>
       <c r="Z32">
         <f t="shared" si="8"/>
-        <v>492.06207264428838</v>
+        <v>643.95606325960682</v>
       </c>
       <c r="AA32">
         <f>Y32/reranking!E32*100</f>
-        <v>29.016685993170437</v>
+        <v>41.7098068984264</v>
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
@@ -8079,15 +8175,15 @@
       </c>
       <c r="K33">
         <f>E33-reranking!E33</f>
-        <v>-197.74999999999909</v>
+        <v>-210.91666666666606</v>
       </c>
       <c r="L33">
         <f t="shared" si="4"/>
-        <v>-19774.999999999909</v>
+        <v>-21091.666666666606</v>
       </c>
       <c r="M33">
         <f>K33/reranking!E33*100</f>
-        <v>-5.8822775202067596</v>
+        <v>-6.2494572093664615</v>
       </c>
       <c r="O33" t="s">
         <v>12</v>
@@ -8119,15 +8215,15 @@
       </c>
       <c r="Y33">
         <f>S33-reranking!E33</f>
-        <v>-184.26436781609209</v>
+        <v>-197.43103448275906</v>
       </c>
       <c r="Z33">
         <f t="shared" si="8"/>
-        <v>-18426.436781609209</v>
+        <v>-19743.103448275906</v>
       </c>
       <c r="AA33">
         <f>Y33/reranking!E33*100</f>
-        <v>-5.4811334947140997</v>
+        <v>-5.8498781594672176</v>
       </c>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
@@ -8161,15 +8257,15 @@
       </c>
       <c r="K34">
         <f>E34-reranking!E34</f>
-        <v>-31.014367816092033</v>
+        <v>-33.086206896551744</v>
       </c>
       <c r="L34">
         <f t="shared" si="4"/>
-        <v>-3101.4367816092035</v>
+        <v>-3308.6206896551744</v>
       </c>
       <c r="M34">
         <f>K34/reranking!E34*100</f>
-        <v>-10.664176744921376</v>
+        <v>-11.296098264478221</v>
       </c>
       <c r="O34" t="s">
         <v>13</v>
@@ -8201,15 +8297,15 @@
       </c>
       <c r="Y34">
         <f>S34-reranking!E34</f>
-        <v>-33.255747126436802</v>
+        <v>-35.327586206896513</v>
       </c>
       <c r="Z34">
         <f t="shared" si="8"/>
-        <v>-3325.57471264368</v>
+        <v>-3532.7586206896513</v>
       </c>
       <c r="AA34">
         <f>Y34/reranking!E34*100</f>
-        <v>-11.434866808947913</v>
+        <v>-12.061336812879539</v>
       </c>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
@@ -8243,15 +8339,15 @@
       </c>
       <c r="K35">
         <f>E35-reranking!E35</f>
-        <v>-228.76436781609345</v>
+        <v>-244.00287356321996</v>
       </c>
       <c r="L35">
         <f t="shared" si="4"/>
-        <v>-22876.436781609344</v>
+        <v>-24400.287356321998</v>
       </c>
       <c r="M35">
         <f>K35/reranking!E35*100</f>
-        <v>-6.263020095790182</v>
+        <v>-6.6524602108248914</v>
       </c>
       <c r="O35" t="s">
         <v>14</v>
@@ -8283,15 +8379,15 @@
       </c>
       <c r="Y35">
         <f>S35-reranking!E35</f>
-        <v>-217.52011494252929</v>
+        <v>-232.7586206896558</v>
       </c>
       <c r="Z35">
         <f t="shared" si="8"/>
-        <v>-21752.011494252929</v>
+        <v>-23275.86206896558</v>
       </c>
       <c r="AA35">
         <f>Y35/reranking!E35*100</f>
-        <v>-5.95517940197246</v>
+        <v>-6.3458984734588828</v>
       </c>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
@@ -8325,15 +8421,15 @@
       </c>
       <c r="K36">
         <f>E36-reranking!E36</f>
-        <v>-1436.6034482758623</v>
+        <v>-1433.9568965517192</v>
       </c>
       <c r="L36">
         <f t="shared" si="4"/>
-        <v>-143660.34482758623</v>
+        <v>-143395.68965517191</v>
       </c>
       <c r="M36">
         <f>K36/reranking!E36*100</f>
-        <v>-9.9050189011198011</v>
+        <v>-9.8885759925047214</v>
       </c>
       <c r="O36" t="s">
         <v>30</v>
@@ -8365,15 +8461,15 @@
       </c>
       <c r="Y36">
         <f>S36-reranking!E36</f>
-        <v>-1438.7758620689674</v>
+        <v>-1436.1293103448243</v>
       </c>
       <c r="Z36">
         <f t="shared" si="8"/>
-        <v>-143877.58620689675</v>
+        <v>-143612.93103448243</v>
       </c>
       <c r="AA36">
         <f>Y36/reranking!E36*100</f>
-        <v>-9.9199971470007942</v>
+        <v>-9.9035569720111081</v>
       </c>
     </row>
     <row r="38" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -8462,33 +8558,39 @@
       <c r="B40">
         <v>0.80783563818411519</v>
       </c>
+      <c r="C40">
+        <v>0.80691956514063767</v>
+      </c>
+      <c r="D40">
+        <v>0.8132572759333393</v>
+      </c>
       <c r="E40">
         <f>AVERAGE(B40:D40)</f>
-        <v>0.80783563818411519</v>
+        <v>0.80933749308603076</v>
       </c>
       <c r="G40">
         <f t="shared" ref="G40:G55" si="10">E40-E3</f>
-        <v>-3.9333904049129176E-3</v>
+        <v>-2.4315355029973507E-3</v>
       </c>
       <c r="H40">
         <f>G40*100</f>
-        <v>-0.39333904049129176</v>
+        <v>-0.24315355029973507</v>
       </c>
       <c r="I40">
         <f t="shared" ref="I40:I55" si="11">G40/E3*100</f>
-        <v>-0.48454551311839511</v>
+        <v>-0.29953538720536194</v>
       </c>
       <c r="K40">
         <f>E40-reranking!E40</f>
-        <v>3.7902300459486504E-2</v>
+        <v>3.7757088724036159E-2</v>
       </c>
       <c r="L40">
         <f>K40*100</f>
-        <v>3.7902300459486504</v>
+        <v>3.7757088724036159</v>
       </c>
       <c r="M40">
         <f>K40/reranking!E40*100</f>
-        <v>4.9228028716743903</v>
+        <v>4.8934742912835878</v>
       </c>
       <c r="N40" t="s">
         <v>22</v>
@@ -8511,44 +8613,44 @@
       </c>
       <c r="U40">
         <f>S40-E40</f>
-        <v>9.5638907530060102E-5</v>
+        <v>-1.4062159943855068E-3</v>
       </c>
       <c r="V40">
         <f>U40*100</f>
-        <v>9.5638907530060102E-3</v>
+        <v>-0.14062159943855068</v>
       </c>
       <c r="W40">
         <f t="shared" ref="W40:W55" si="12">U40/E41*100</f>
-        <v>1.2533360881363554E-2</v>
+        <v>-0.18333930666730805</v>
       </c>
       <c r="X40" t="s">
         <v>22</v>
       </c>
       <c r="Y40">
         <f>S40-reranking!E40</f>
-        <v>3.7997939367016564E-2</v>
+        <v>3.6350872729650652E-2</v>
       </c>
       <c r="Z40">
         <f>Y40*100</f>
-        <v>3.7997939367016564</v>
+        <v>3.6350872729650652</v>
       </c>
       <c r="AA40">
         <f>Y40/reranking!E40*100</f>
-        <v>4.9352245844180809</v>
+        <v>4.7112229035557878</v>
       </c>
       <c r="AB40" t="s">
         <v>22</v>
       </c>
       <c r="AD40">
         <f t="shared" ref="AD40:AD55" si="13">AA40-AA21</f>
-        <v>-3.7829813021326943</v>
+        <v>-2.2702792478658713</v>
       </c>
       <c r="AE40" t="s">
         <v>26</v>
       </c>
       <c r="AG40">
         <f>AD41</f>
-        <v>3.916063566818198</v>
+        <v>5.1977877559939092</v>
       </c>
       <c r="AH40" t="s">
         <v>22</v>
@@ -8561,33 +8663,39 @@
       <c r="B41">
         <v>0.7630747126436781</v>
       </c>
+      <c r="C41">
+        <v>0.76594827586206893</v>
+      </c>
+      <c r="D41">
+        <v>0.77198275862068966</v>
+      </c>
       <c r="E41">
         <f t="shared" ref="E41:E55" si="14">AVERAGE(B41:D41)</f>
-        <v>0.7630747126436781</v>
+        <v>0.76700191570881227</v>
       </c>
       <c r="G41">
         <f t="shared" si="10"/>
-        <v>8.40311986863711E-2</v>
+        <v>8.7958401751505266E-2</v>
       </c>
       <c r="H41">
         <f t="shared" ref="H41:H55" si="15">G41*100</f>
-        <v>8.4031198686371091</v>
+        <v>8.7958401751505271</v>
       </c>
       <c r="I41">
         <f t="shared" si="11"/>
-        <v>12.374935767614788</v>
+        <v>12.95327912623806</v>
       </c>
       <c r="K41">
         <f>E41-reranking!E41</f>
-        <v>5.6224253161639703E-2</v>
+        <v>6.2275900479167201E-2</v>
       </c>
       <c r="L41">
         <f t="shared" ref="L41:L55" si="16">K41*100</f>
-        <v>5.6224253161639703</v>
+        <v>6.2275900479167206</v>
       </c>
       <c r="M41">
         <f>K41/reranking!E41*100</f>
-        <v>7.9541934800239602</v>
+        <v>8.8368953512910569</v>
       </c>
       <c r="N41" t="s">
         <v>22</v>
@@ -8610,44 +8718,44 @@
       </c>
       <c r="U41">
         <f t="shared" ref="U41:U55" si="18">S41-E41</f>
-        <v>5.5281882868090104E-3</v>
+        <v>1.6009852216748444E-3</v>
       </c>
       <c r="V41">
         <f t="shared" ref="V41:V55" si="19">U41*100</f>
-        <v>0.55281882868090104</v>
+        <v>0.16009852216748444</v>
       </c>
       <c r="W41">
         <f t="shared" si="12"/>
-        <v>0.78978171043167045</v>
+        <v>0.22654734743777349</v>
       </c>
       <c r="X41" t="s">
         <v>22</v>
       </c>
       <c r="Y41">
         <f>S41-reranking!E41</f>
-        <v>6.1752441448448714E-2</v>
+        <v>6.3876885700842045E-2</v>
       </c>
       <c r="Z41">
         <f t="shared" ref="Z41:Z55" si="20">Y41*100</f>
-        <v>6.1752441448448714</v>
+        <v>6.3876885700842045</v>
       </c>
       <c r="AA41">
         <f>Y41/reranking!E41*100</f>
-        <v>8.7362808667761627</v>
+        <v>9.0640737421942408</v>
       </c>
       <c r="AB41" t="s">
         <v>22</v>
       </c>
       <c r="AD41">
         <f t="shared" si="13"/>
-        <v>3.916063566818198</v>
+        <v>5.1977877559939092</v>
       </c>
       <c r="AE41" t="s">
         <v>22</v>
       </c>
       <c r="AG41">
         <f>AD42</f>
-        <v>-5.5212495751462232</v>
+        <v>-5.6233696090730518</v>
       </c>
       <c r="AH41" t="s">
         <v>26</v>
@@ -8660,33 +8768,39 @@
       <c r="B42">
         <v>0.69996408042767566</v>
       </c>
+      <c r="C42">
+        <v>0.70626197314811712</v>
+      </c>
+      <c r="D42">
+        <v>0.71384099613608976</v>
+      </c>
       <c r="E42">
         <f t="shared" si="14"/>
-        <v>0.69996408042767566</v>
+        <v>0.70668901657062755</v>
       </c>
       <c r="G42">
         <f t="shared" si="10"/>
-        <v>4.9692688375222116E-2</v>
+        <v>5.6417624518174003E-2</v>
       </c>
       <c r="H42">
         <f t="shared" si="15"/>
-        <v>4.9692688375222112</v>
+        <v>5.6417624518174003</v>
       </c>
       <c r="I42">
         <f t="shared" si="11"/>
-        <v>7.6418383128276535</v>
+        <v>8.6760120786035024</v>
       </c>
       <c r="K42">
         <f>E42-reranking!E42</f>
-        <v>-2.5265388142427958E-2</v>
+        <v>-2.636161086384925E-2</v>
       </c>
       <c r="L42">
         <f t="shared" si="16"/>
-        <v>-2.5265388142427958</v>
+        <v>-2.636161086384925</v>
       </c>
       <c r="M42">
         <f>K42/reranking!E42*100</f>
-        <v>-3.4837784780370797</v>
+        <v>-3.596151463113721</v>
       </c>
       <c r="O42" t="s">
         <v>2</v>
@@ -8706,44 +8820,44 @@
       </c>
       <c r="U42">
         <f t="shared" si="18"/>
-        <v>9.2672413785749308E-3</v>
+        <v>2.5423052356230436E-3</v>
       </c>
       <c r="V42">
         <f t="shared" si="19"/>
-        <v>0.92672413785749308</v>
+        <v>0.25423052356230436</v>
       </c>
       <c r="W42">
         <f t="shared" si="12"/>
-        <v>1.1635075006580398</v>
+        <v>0.31918788879808813</v>
       </c>
       <c r="X42" t="s">
         <v>22</v>
       </c>
       <c r="Y42">
         <f>S42-reranking!E42</f>
-        <v>-1.5998146763853027E-2</v>
+        <v>-2.3819305628226206E-2</v>
       </c>
       <c r="Z42">
         <f t="shared" si="20"/>
-        <v>-1.5998146763853027</v>
+        <v>-2.3819305628226206</v>
       </c>
       <c r="AA42">
         <f>Y42/reranking!E42*100</f>
-        <v>-2.2059427336006801</v>
+        <v>-3.2493397777434243</v>
       </c>
       <c r="AB42" t="s">
         <v>26</v>
       </c>
       <c r="AD42">
         <f t="shared" si="13"/>
-        <v>-5.5212495751462232</v>
+        <v>-5.6233696090730518</v>
       </c>
       <c r="AE42" t="s">
         <v>26</v>
       </c>
       <c r="AG42">
         <f>AD44</f>
-        <v>7.6964858984874773</v>
+        <v>5.3944469436855282</v>
       </c>
       <c r="AH42" t="s">
         <v>22</v>
@@ -8756,6 +8870,12 @@
       <c r="B43">
         <v>0.7964917607607771</v>
       </c>
+      <c r="C43">
+        <v>0.7964917607607771</v>
+      </c>
+      <c r="D43">
+        <v>0.7964917607607771</v>
+      </c>
       <c r="E43">
         <f t="shared" si="14"/>
         <v>0.7964917607607771</v>
@@ -8774,15 +8894,15 @@
       </c>
       <c r="K43">
         <f>E43-reranking!E43</f>
-        <v>9.2651624930237819E-3</v>
+        <v>9.6284092283113187E-3</v>
       </c>
       <c r="L43">
         <f t="shared" si="16"/>
-        <v>0.92651624930237819</v>
+        <v>0.96284092283113187</v>
       </c>
       <c r="M43">
         <f>K43/reranking!E43*100</f>
-        <v>1.1769371758285654</v>
+        <v>1.2236443862278485</v>
       </c>
       <c r="O43" t="s">
         <v>3</v>
@@ -8810,26 +8930,26 @@
       </c>
       <c r="W43">
         <f t="shared" si="12"/>
-        <v>-0.12108620934999578</v>
+        <v>-0.11691968685362573</v>
       </c>
       <c r="Y43">
         <f>S43-reranking!E43</f>
-        <v>8.8817552544868672E-3</v>
+        <v>9.245001989774404E-3</v>
       </c>
       <c r="Z43">
         <f t="shared" si="20"/>
-        <v>0.88817552544868672</v>
+        <v>0.9245001989774404</v>
       </c>
       <c r="AA43">
         <f>Y43/reranking!E43*100</f>
-        <v>1.1282336336234899</v>
+        <v>1.174918360572923</v>
       </c>
       <c r="AB43" t="s">
         <v>22</v>
       </c>
       <c r="AD43">
         <f t="shared" si="13"/>
-        <v>-0.12584985150493466</v>
+        <v>-9.0132261555081028E-2</v>
       </c>
       <c r="AG43">
         <f>AD49</f>
@@ -8846,33 +8966,39 @@
       <c r="B44">
         <v>0.31663988871654941</v>
       </c>
+      <c r="C44">
+        <v>0.33960651241618589</v>
+      </c>
+      <c r="D44">
+        <v>0.32752437910441268</v>
+      </c>
       <c r="E44">
         <f t="shared" si="14"/>
-        <v>0.31663988871654941</v>
+        <v>0.3279235934123827</v>
       </c>
       <c r="G44">
         <f t="shared" si="10"/>
-        <v>3.9810151324936427E-2</v>
+        <v>5.1093856020769712E-2</v>
       </c>
       <c r="H44">
         <f t="shared" si="15"/>
-        <v>3.9810151324936429</v>
+        <v>5.109385602076971</v>
       </c>
       <c r="I44">
         <f t="shared" si="11"/>
-        <v>14.380735140683099</v>
+        <v>18.456780150208559</v>
       </c>
       <c r="K44">
         <f>E44-reranking!E44</f>
-        <v>3.8698712293601834E-2</v>
+        <v>4.6448640364930349E-2</v>
       </c>
       <c r="L44">
         <f t="shared" si="16"/>
-        <v>3.8698712293601831</v>
+        <v>4.6448640364930345</v>
       </c>
       <c r="M44">
         <f>K44/reranking!E44*100</f>
-        <v>13.923346224423177</v>
+        <v>16.501873385906499</v>
       </c>
       <c r="N44" t="s">
         <v>22</v>
@@ -8895,37 +9021,37 @@
       </c>
       <c r="U44">
         <f t="shared" si="18"/>
-        <v>1.4682688514277731E-2</v>
+        <v>3.3989838184444454E-3</v>
       </c>
       <c r="V44">
         <f t="shared" si="19"/>
-        <v>1.4682688514277731</v>
+        <v>0.33989838184444454</v>
       </c>
       <c r="W44">
         <f t="shared" si="12"/>
-        <v>2.013568765052355</v>
+        <v>0.4641386146635022</v>
       </c>
       <c r="X44" t="s">
         <v>22</v>
       </c>
       <c r="Y44">
         <f>S44-reranking!E44</f>
-        <v>5.3381400807879564E-2</v>
+        <v>4.9847624183374795E-2</v>
       </c>
       <c r="Z44">
         <f t="shared" si="20"/>
-        <v>5.3381400807879569</v>
+        <v>4.9847624183374792</v>
       </c>
       <c r="AA44">
         <f>Y44/reranking!E44*100</f>
-        <v>19.206006643164027</v>
+        <v>17.70943511800542</v>
       </c>
       <c r="AB44" t="s">
         <v>22</v>
       </c>
       <c r="AD44">
         <f t="shared" si="13"/>
-        <v>7.6964858984874773</v>
+        <v>5.3944469436855282</v>
       </c>
       <c r="AE44" t="s">
         <v>22</v>
@@ -8942,33 +9068,39 @@
       <c r="B45">
         <v>0.72918733986698314</v>
       </c>
+      <c r="C45">
+        <v>0.73067953071328751</v>
+      </c>
+      <c r="D45">
+        <v>0.73709566026325046</v>
+      </c>
       <c r="E45">
         <f t="shared" si="14"/>
-        <v>0.72918733986698314</v>
+        <v>0.73232084361450711</v>
       </c>
       <c r="G45">
         <f t="shared" si="10"/>
-        <v>-3.1732758609365419E-2</v>
+        <v>-2.859925486184145E-2</v>
       </c>
       <c r="H45">
         <f t="shared" si="15"/>
-        <v>-3.1732758609365419</v>
+        <v>-2.859925486184145</v>
       </c>
       <c r="I45">
         <f t="shared" si="11"/>
-        <v>-4.1703141595164164</v>
+        <v>-3.7585095884716457</v>
       </c>
       <c r="K45">
         <f>E45-reranking!E45</f>
-        <v>2.2632017650869751E-2</v>
+        <v>2.3309293267555709E-2</v>
       </c>
       <c r="L45">
         <f t="shared" si="16"/>
-        <v>2.2632017650869751</v>
+        <v>2.3309293267555709</v>
       </c>
       <c r="M45">
         <f>K45/reranking!E45*100</f>
-        <v>3.203148704603108</v>
+        <v>3.2875759578457382</v>
       </c>
       <c r="N45" t="s">
         <v>22</v>
@@ -8991,37 +9123,37 @@
       </c>
       <c r="U45">
         <f t="shared" si="18"/>
-        <v>-2.9746568854567279E-3</v>
+        <v>-6.108160632980697E-3</v>
       </c>
       <c r="V45">
         <f t="shared" si="19"/>
-        <v>-0.29746568854567279</v>
+        <v>-0.6108160632980697</v>
       </c>
       <c r="W45">
         <f t="shared" si="12"/>
-        <v>-0.96949009661388286</v>
+        <v>-1.9907510244807074</v>
       </c>
       <c r="X45" t="s">
         <v>26</v>
       </c>
       <c r="Y45">
         <f>S45-reranking!E45</f>
-        <v>1.9657360765413023E-2</v>
+        <v>1.7201132634575012E-2</v>
       </c>
       <c r="Z45">
         <f t="shared" si="20"/>
-        <v>1.9657360765413023</v>
+        <v>1.7201132634575012</v>
       </c>
       <c r="AA45">
         <f>Y45/reranking!E45*100</f>
-        <v>2.7821403572133088</v>
+        <v>2.426072272892835</v>
       </c>
       <c r="AB45" t="s">
         <v>22</v>
       </c>
       <c r="AD45">
         <f t="shared" si="13"/>
-        <v>-8.0132142187352855</v>
+        <v>-7.4073557959747607</v>
       </c>
       <c r="AE45" t="s">
         <v>26</v>
@@ -9034,6 +9166,12 @@
       <c r="B46">
         <v>0.30682694911956793</v>
       </c>
+      <c r="C46">
+        <v>0.30682694911956793</v>
+      </c>
+      <c r="D46">
+        <v>0.30682694911956793</v>
+      </c>
       <c r="E46">
         <f t="shared" si="14"/>
         <v>0.30682694911956793</v>
@@ -9052,15 +9190,15 @@
       </c>
       <c r="K46">
         <f>E46-reranking!E46</f>
-        <v>2.6673585176467951E-2</v>
+        <v>2.7089238166809138E-2</v>
       </c>
       <c r="L46">
         <f t="shared" si="16"/>
-        <v>2.6673585176467949</v>
+        <v>2.7089238166809135</v>
       </c>
       <c r="M46">
         <f>K46/reranking!E46*100</f>
-        <v>9.5210654625176812</v>
+        <v>9.6837991826507377</v>
       </c>
       <c r="N46" t="s">
         <v>22</v>
@@ -9098,22 +9236,22 @@
       </c>
       <c r="Y46">
         <f>S46-reranking!E46</f>
-        <v>2.3543089628219604E-2</v>
+        <v>2.3958742618560791E-2</v>
       </c>
       <c r="Z46">
         <f t="shared" si="20"/>
-        <v>2.3543089628219604</v>
+        <v>2.3958742618560791</v>
       </c>
       <c r="AA46">
         <f>Y46/reranking!E46*100</f>
-        <v>8.4036433819160852</v>
+        <v>8.5647167616263467</v>
       </c>
       <c r="AB46" t="s">
         <v>22</v>
       </c>
       <c r="AD46">
         <f t="shared" si="13"/>
-        <v>0.52517180754656678</v>
+        <v>0.64475042671137928</v>
       </c>
       <c r="AG46" t="s">
         <v>53</v>
@@ -9126,6 +9264,12 @@
       <c r="B47">
         <v>0.23263862729072571</v>
       </c>
+      <c r="C47">
+        <v>0.23263862729072571</v>
+      </c>
+      <c r="D47">
+        <v>0.23263862729072571</v>
+      </c>
       <c r="E47">
         <f t="shared" si="14"/>
         <v>0.23263862729072571</v>
@@ -9144,15 +9288,15 @@
       </c>
       <c r="K47">
         <f>E47-reranking!E47</f>
-        <v>2.9932826757431003E-2</v>
+        <v>3.0556504925092015E-2</v>
       </c>
       <c r="L47">
         <f t="shared" si="16"/>
-        <v>2.9932826757431004</v>
+        <v>3.0556504925092014</v>
       </c>
       <c r="M47">
         <f>K47/reranking!E47*100</f>
-        <v>14.766635527291927</v>
+        <v>15.12083531555807</v>
       </c>
       <c r="N47" t="s">
         <v>22</v>
@@ -9190,22 +9334,22 @@
       </c>
       <c r="Y47">
         <f>S47-reranking!E47</f>
-        <v>2.0672544836997986E-2</v>
+        <v>2.1296223004658998E-2</v>
       </c>
       <c r="Z47">
         <f t="shared" si="20"/>
-        <v>2.0672544836997986</v>
+        <v>2.1296223004658996</v>
       </c>
       <c r="AA47">
         <f>Y47/reranking!E47*100</f>
-        <v>10.198299596070262</v>
+        <v>10.538400307438902</v>
       </c>
       <c r="AB47" t="s">
         <v>22</v>
       </c>
       <c r="AD47">
         <f t="shared" si="13"/>
-        <v>-6.4100358067238385</v>
+        <v>-6.2260992251109322</v>
       </c>
       <c r="AE47" t="s">
         <v>26</v>
@@ -9215,7 +9359,7 @@
       </c>
       <c r="AG47">
         <f>AD40</f>
-        <v>-3.7829813021326943</v>
+        <v>-2.2702792478658713</v>
       </c>
       <c r="AH47" t="s">
         <v>26</v>
@@ -9228,6 +9372,12 @@
       <c r="B48">
         <v>0.38350716233253479</v>
       </c>
+      <c r="C48">
+        <v>0.38350716233253479</v>
+      </c>
+      <c r="D48">
+        <v>0.38350716233253479</v>
+      </c>
       <c r="E48">
         <f t="shared" si="14"/>
         <v>0.38350716233253479</v>
@@ -9246,15 +9396,15 @@
       </c>
       <c r="K48">
         <f>E48-reranking!E48</f>
-        <v>2.2362172603607178E-2</v>
+        <v>2.2567729155222593E-2</v>
       </c>
       <c r="L48">
         <f t="shared" si="16"/>
-        <v>2.2362172603607178</v>
+        <v>2.2567729155222596</v>
       </c>
       <c r="M48">
         <f>K48/reranking!E48*100</f>
-        <v>6.192020722865915</v>
+        <v>6.2524975330518</v>
       </c>
       <c r="N48" t="s">
         <v>22</v>
@@ -9292,22 +9442,22 @@
       </c>
       <c r="Y48">
         <f>S48-reranking!E48</f>
-        <v>2.5778144598007202E-2</v>
+        <v>2.5983701149622618E-2</v>
       </c>
       <c r="Z48">
         <f t="shared" si="20"/>
-        <v>2.5778144598007202</v>
+        <v>2.598370114962262</v>
       </c>
       <c r="AA48">
         <f>Y48/reranking!E48*100</f>
-        <v>7.1378934586233802</v>
+        <v>7.1989089473795662</v>
       </c>
       <c r="AB48" t="s">
         <v>22</v>
       </c>
       <c r="AD48">
         <f t="shared" si="13"/>
-        <v>4.1649745511730814</v>
+        <v>4.2407263518696006</v>
       </c>
       <c r="AE48" t="s">
         <v>22</v>
@@ -9317,7 +9467,7 @@
       </c>
       <c r="AG48">
         <f>AD43</f>
-        <v>-0.12584985150493466</v>
+        <v>-9.0132261555081028E-2</v>
       </c>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
@@ -9327,6 +9477,12 @@
       <c r="B49">
         <v>0.4653735632183908</v>
       </c>
+      <c r="C49">
+        <v>0.4653735632183908</v>
+      </c>
+      <c r="D49">
+        <v>0.4653735632183908</v>
+      </c>
       <c r="E49">
         <f t="shared" si="14"/>
         <v>0.4653735632183908</v>
@@ -9413,7 +9569,7 @@
       </c>
       <c r="AG49">
         <f>AD45</f>
-        <v>-8.0132142187352855</v>
+        <v>-7.4073557959747607</v>
       </c>
       <c r="AH49" t="s">
         <v>26</v>
@@ -9426,6 +9582,12 @@
       <c r="B50">
         <v>0.62931034482758619</v>
       </c>
+      <c r="C50">
+        <v>0.62931034482758619</v>
+      </c>
+      <c r="D50">
+        <v>0.62931034482758619</v>
+      </c>
       <c r="E50">
         <f t="shared" si="14"/>
         <v>0.62931034482758619</v>
@@ -9512,7 +9674,7 @@
       </c>
       <c r="AG50">
         <f>AD46</f>
-        <v>0.52517180754656678</v>
+        <v>0.64475042671137928</v>
       </c>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
@@ -9522,33 +9684,39 @@
       <c r="B51">
         <v>15.26280314757906</v>
       </c>
+      <c r="C51">
+        <v>18.702104985713959</v>
+      </c>
+      <c r="D51">
+        <v>16.484393389060578</v>
+      </c>
       <c r="E51">
         <f t="shared" si="14"/>
-        <v>15.26280314757906</v>
+        <v>16.816433840784534</v>
       </c>
       <c r="G51">
         <f t="shared" si="10"/>
-        <v>-1.0955383537829633</v>
+        <v>0.45809233942251026</v>
       </c>
       <c r="H51">
         <f t="shared" si="15"/>
-        <v>-109.55383537829633</v>
+        <v>45.809233942251026</v>
       </c>
       <c r="I51">
         <f t="shared" si="11"/>
-        <v>-6.6971236276718331</v>
+        <v>2.8003593113908809</v>
       </c>
       <c r="K51">
         <f>E51-reranking!E51</f>
-        <v>-0.12097382956537928</v>
+        <v>1.4153361649348799</v>
       </c>
       <c r="L51">
         <f t="shared" si="16"/>
-        <v>-12.097382956537928</v>
+        <v>141.53361649348798</v>
       </c>
       <c r="M51">
         <f>K51/reranking!E51*100</f>
-        <v>-0.78637274672604263</v>
+        <v>9.1898395473087486</v>
       </c>
       <c r="O51" t="s">
         <v>11</v>
@@ -9568,31 +9736,31 @@
       </c>
       <c r="U51">
         <f t="shared" si="18"/>
-        <v>2.2102848332503768</v>
+        <v>0.6566541400449033</v>
       </c>
       <c r="V51">
         <f t="shared" si="19"/>
-        <v>221.02848332503768</v>
+        <v>65.66541400449033</v>
       </c>
       <c r="W51">
         <f t="shared" si="12"/>
-        <v>7.0844224314000892E-2</v>
+        <v>2.1047130439585643E-2</v>
       </c>
       <c r="Y51">
         <f>S51-reranking!E51</f>
-        <v>2.0893110036849976</v>
+        <v>2.0719903049797832</v>
       </c>
       <c r="Z51">
         <f t="shared" si="20"/>
-        <v>208.93110036849976</v>
+        <v>207.19903049797833</v>
       </c>
       <c r="AA51">
         <f>Y51/reranking!E51*100</f>
-        <v>13.581261654982852</v>
+        <v>13.453523564290199</v>
       </c>
       <c r="AD51">
         <f t="shared" si="13"/>
-        <v>-15.435424338187586</v>
+        <v>-28.256283334136199</v>
       </c>
       <c r="AE51" t="s">
         <v>22</v>
@@ -9602,7 +9770,7 @@
       </c>
       <c r="AG51">
         <f t="shared" ref="AG51:AG52" si="21">AD47</f>
-        <v>-6.4100358067238385</v>
+        <v>-6.2260992251109322</v>
       </c>
       <c r="AH51" t="s">
         <v>26</v>
@@ -9615,6 +9783,12 @@
       <c r="B52">
         <v>3119.9224137931028</v>
       </c>
+      <c r="C52">
+        <v>3119.9224137931028</v>
+      </c>
+      <c r="D52">
+        <v>3119.9224137931028</v>
+      </c>
       <c r="E52">
         <f t="shared" si="14"/>
         <v>3119.9224137931028</v>
@@ -9633,15 +9807,15 @@
       </c>
       <c r="K52">
         <f>E52-reranking!E52</f>
-        <v>-270.05172413793116</v>
+        <v>-269.47126436781627</v>
       </c>
       <c r="L52">
         <f t="shared" si="16"/>
-        <v>-27005.172413793116</v>
+        <v>-26947.126436781626</v>
       </c>
       <c r="M52">
         <f>K52/reranking!E52*100</f>
-        <v>-7.96618832917554</v>
+        <v>-7.9504268301471264</v>
       </c>
       <c r="N52" t="s">
         <v>22</v>
@@ -9676,26 +9850,26 @@
       </c>
       <c r="Y52">
         <f>S52-reranking!E52</f>
-        <v>-269.67241379310281</v>
+        <v>-269.09195402298792</v>
       </c>
       <c r="Z52">
         <f t="shared" si="20"/>
-        <v>-26967.241379310282</v>
+        <v>-26909.195402298792</v>
       </c>
       <c r="AA52">
         <f>Y52/reranking!E52*100</f>
-        <v>-7.9549991480964231</v>
+        <v>-7.9392357328345788</v>
       </c>
       <c r="AD52">
         <f t="shared" si="13"/>
-        <v>-2.4738656533823233</v>
+        <v>-2.0893575733673613</v>
       </c>
       <c r="AF52" t="s">
         <v>58</v>
       </c>
       <c r="AG52">
         <f t="shared" si="21"/>
-        <v>4.1649745511730814</v>
+        <v>4.2407263518696006</v>
       </c>
       <c r="AH52" t="s">
         <v>22</v>
@@ -9708,6 +9882,12 @@
       <c r="B53">
         <v>253.4568965517241</v>
       </c>
+      <c r="C53">
+        <v>253.4568965517241</v>
+      </c>
+      <c r="D53">
+        <v>253.4568965517241</v>
+      </c>
       <c r="E53">
         <f t="shared" si="14"/>
         <v>253.4568965517241</v>
@@ -9726,15 +9906,15 @@
       </c>
       <c r="K53">
         <f>E53-reranking!E53</f>
-        <v>-22.456896551724213</v>
+        <v>-22.704022988505841</v>
       </c>
       <c r="L53">
         <f t="shared" si="16"/>
-        <v>-2245.6896551724212</v>
+        <v>-2270.402298850584</v>
       </c>
       <c r="M53">
         <f>K53/reranking!E53*100</f>
-        <v>-8.1390989189527225</v>
+        <v>-8.2213019229168722</v>
       </c>
       <c r="N53" t="s">
         <v>22</v>
@@ -9765,23 +9945,23 @@
       </c>
       <c r="W53">
         <f t="shared" si="12"/>
-        <v>0.18961851412683672</v>
+        <v>0.1896185141268367</v>
       </c>
       <c r="Y53">
         <f>S53-reranking!E53</f>
-        <v>-16.060344827586221</v>
+        <v>-16.307471264367848</v>
       </c>
       <c r="Z53">
         <f t="shared" si="20"/>
-        <v>-1606.0344827586221</v>
+        <v>-1630.7471264367848</v>
       </c>
       <c r="AA53">
         <f>Y53/reranking!E53*100</f>
-        <v>-5.8207836030744273</v>
+        <v>-5.9050611837176499</v>
       </c>
       <c r="AD53">
         <f t="shared" si="13"/>
-        <v>5.6140832058734853</v>
+        <v>6.1562756291618888</v>
       </c>
     </row>
     <row r="54" spans="1:34" x14ac:dyDescent="0.25">
@@ -9791,33 +9971,39 @@
       <c r="B54">
         <v>3373.379310344827</v>
       </c>
+      <c r="C54">
+        <v>3373.379310344827</v>
+      </c>
+      <c r="D54">
+        <v>3373.379310344827</v>
+      </c>
       <c r="E54">
         <f t="shared" si="14"/>
-        <v>3373.379310344827</v>
+        <v>3373.3793103448274</v>
       </c>
       <c r="G54">
         <f t="shared" si="10"/>
-        <v>-38.212643678161385</v>
+        <v>-38.21264367816093</v>
       </c>
       <c r="H54">
         <f t="shared" si="15"/>
-        <v>-3821.2643678161385</v>
+        <v>-3821.264367816093</v>
       </c>
       <c r="I54">
         <f t="shared" si="11"/>
-        <v>-1.1200824774223246</v>
+        <v>-1.1200824774223115</v>
       </c>
       <c r="K54">
         <f>E54-reranking!E54</f>
-        <v>-292.5086206896558</v>
+        <v>-292.17528735632231</v>
       </c>
       <c r="L54">
         <f t="shared" si="16"/>
-        <v>-29250.86206896558</v>
+        <v>-29217.52873563223</v>
       </c>
       <c r="M54">
         <f>K54/reranking!E54*100</f>
-        <v>-7.9792024795234893</v>
+        <v>-7.9708344145128782</v>
       </c>
       <c r="N54" t="s">
         <v>22</v>
@@ -9840,31 +10026,31 @@
       </c>
       <c r="U54">
         <f t="shared" si="18"/>
-        <v>6.7758620689660347</v>
+        <v>6.77586206896558</v>
       </c>
       <c r="V54">
         <f t="shared" si="19"/>
-        <v>677.58620689660347</v>
+        <v>677.586206896558</v>
       </c>
       <c r="W54">
         <f t="shared" si="12"/>
-        <v>6.1532584086707691E-2</v>
+        <v>6.1532584086703562E-2</v>
       </c>
       <c r="Y54">
         <f>S54-reranking!E54</f>
-        <v>-285.73275862068976</v>
+        <v>-285.39942528735673</v>
       </c>
       <c r="Z54">
         <f t="shared" si="20"/>
-        <v>-28573.275862068978</v>
+        <v>-28539.942528735672</v>
       </c>
       <c r="AA54">
         <f>Y54/reranking!E54*100</f>
-        <v>-7.7943669854647846</v>
+        <v>-7.7859821121296307</v>
       </c>
       <c r="AD54">
         <f t="shared" si="13"/>
-        <v>-1.8391875834923246</v>
+        <v>-1.4400836386707478</v>
       </c>
       <c r="AG54" t="s">
         <v>59</v>
@@ -9877,6 +10063,12 @@
       <c r="B55">
         <v>11011.8275862069</v>
       </c>
+      <c r="C55">
+        <v>11011.8275862069</v>
+      </c>
+      <c r="D55">
+        <v>11011.8275862069</v>
+      </c>
       <c r="E55">
         <f t="shared" si="14"/>
         <v>11011.8275862069</v>
@@ -9895,15 +10087,15 @@
       </c>
       <c r="K55">
         <f>E55-reranking!E55</f>
-        <v>-1636.7586206896503</v>
+        <v>-1637.4626436781582</v>
       </c>
       <c r="L55">
         <f t="shared" si="16"/>
-        <v>-163675.86206896504</v>
+        <v>-163746.26436781581</v>
       </c>
       <c r="M55">
         <f>K55/reranking!E55*100</f>
-        <v>-12.940249557671665</v>
+        <v>-12.945095052127975</v>
       </c>
       <c r="N55" t="s">
         <v>22</v>
@@ -9938,26 +10130,26 @@
       </c>
       <c r="Y55">
         <f>S55-reranking!E55</f>
-        <v>-1636.7586206896503</v>
+        <v>-1637.4626436781582</v>
       </c>
       <c r="Z55">
         <f t="shared" si="20"/>
-        <v>-163675.86206896504</v>
+        <v>-163746.26436781581</v>
       </c>
       <c r="AA55">
         <f>Y55/reranking!E55*100</f>
-        <v>-12.940249557671665</v>
+        <v>-12.945095052127975</v>
       </c>
       <c r="AD55">
         <f t="shared" si="13"/>
-        <v>-3.0202524106708708</v>
+        <v>-3.041538080116867</v>
       </c>
       <c r="AF55" t="s">
         <v>60</v>
       </c>
       <c r="AG55">
         <f>AD51</f>
-        <v>-15.435424338187586</v>
+        <v>-28.256283334136199</v>
       </c>
       <c r="AH55" t="s">
         <v>22</v>
@@ -9969,7 +10161,7 @@
       </c>
       <c r="AG56">
         <f t="shared" ref="AG56:AG59" si="22">AD52</f>
-        <v>-2.4738656533823233</v>
+        <v>-2.0893575733673613</v>
       </c>
       <c r="AH56" t="s">
         <v>22</v>
@@ -9981,7 +10173,7 @@
       </c>
       <c r="AG57">
         <f t="shared" si="22"/>
-        <v>5.6140832058734853</v>
+        <v>6.1562756291618888</v>
       </c>
       <c r="AH57" t="s">
         <v>26</v>
@@ -9989,20 +10181,23 @@
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
       <c r="AF58" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AG58">
         <f t="shared" si="22"/>
-        <v>-1.8391875834923246</v>
+        <v>-1.4400836386707478</v>
       </c>
       <c r="AH58" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF59" t="s">
+        <v>63</v>
+      </c>
       <c r="AG59">
         <f t="shared" si="22"/>
-        <v>-3.0202524106708708</v>
+        <v>-3.041538080116867</v>
       </c>
       <c r="AH59" t="s">
         <v>22</v>
@@ -10330,21 +10525,27 @@
       <c r="B21">
         <v>0.82311550057741301</v>
       </c>
+      <c r="C21">
+        <v>0.83980886100748964</v>
+      </c>
+      <c r="D21">
+        <v>0.8465087271426881</v>
+      </c>
       <c r="E21">
         <f>AVERAGE(B21:D21)</f>
-        <v>0.82311550057741301</v>
+        <v>0.83647769624253032</v>
       </c>
       <c r="G21">
         <f>E21-E3</f>
-        <v>1.1346471988384899E-2</v>
+        <v>2.4708667653502214E-2</v>
       </c>
       <c r="H21">
         <f>G21*100</f>
-        <v>1.1346471988384899</v>
+        <v>2.4708667653502214</v>
       </c>
       <c r="I21">
         <f>G21/E3*100</f>
-        <v>1.3977463525686249</v>
+        <v>3.0438051691192811</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -10354,21 +10555,27 @@
       <c r="B22">
         <v>0.79784482758620701</v>
       </c>
+      <c r="C22">
+        <v>0.81005747126436778</v>
+      </c>
+      <c r="D22">
+        <v>0.80761494252873567</v>
+      </c>
       <c r="E22">
         <f t="shared" ref="E22:E36" si="0">AVERAGE(B22:D22)</f>
-        <v>0.79784482758620701</v>
+        <v>0.80517241379310345</v>
       </c>
       <c r="G22">
         <f t="shared" ref="G22:G36" si="1">E22-E4</f>
-        <v>0.11880131362890001</v>
+        <v>0.12612889983579645</v>
       </c>
       <c r="H22">
         <f t="shared" ref="H22:H36" si="2">G22*100</f>
-        <v>11.880131362890001</v>
+        <v>12.612889983579645</v>
       </c>
       <c r="I22">
         <f t="shared" ref="I22:I36" si="3">G22/E4*100</f>
-        <v>17.495390381767098</v>
+        <v>18.574494453344627</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -10378,21 +10585,27 @@
       <c r="B23">
         <v>0.81475095782279383</v>
       </c>
+      <c r="C23">
+        <v>0.81945641759132681</v>
+      </c>
+      <c r="D23">
+        <v>0.83251915705489432</v>
+      </c>
       <c r="E23">
         <f t="shared" si="0"/>
-        <v>0.81475095782279383</v>
+        <v>0.82224217748967166</v>
       </c>
       <c r="G23">
         <f t="shared" si="1"/>
-        <v>0.16447956577034029</v>
+        <v>0.17197078543721811</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
-        <v>16.447956577034027</v>
+        <v>17.197078543721812</v>
       </c>
       <c r="I23">
         <f t="shared" si="3"/>
-        <v>25.293987676621132</v>
+        <v>26.446002013778617</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -10402,21 +10615,27 @@
       <c r="B24">
         <v>0.78888568494846134</v>
       </c>
+      <c r="C24">
+        <v>0.78895270744514867</v>
+      </c>
+      <c r="D24">
+        <v>0.78856235040737155</v>
+      </c>
       <c r="E24">
         <f t="shared" si="0"/>
-        <v>0.78888568494846134</v>
+        <v>0.78880024760032708</v>
       </c>
       <c r="G24">
         <f t="shared" si="1"/>
-        <v>4.9154028183192588E-3</v>
+        <v>4.8299654701849937E-3</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
-        <v>0.49154028183192588</v>
+        <v>0.48299654701849937</v>
       </c>
       <c r="I24">
         <f t="shared" si="3"/>
-        <v>0.62698841146931172</v>
+        <v>0.61609037743897554</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -10426,21 +10645,27 @@
       <c r="B25">
         <v>0.33261798698418632</v>
       </c>
+      <c r="C25">
+        <v>0.32460873406107821</v>
+      </c>
+      <c r="D25">
+        <v>0.33347112585562028</v>
+      </c>
       <c r="E25">
         <f t="shared" si="0"/>
-        <v>0.33261798698418632</v>
+        <v>0.33023261563362821</v>
       </c>
       <c r="G25">
         <f t="shared" si="1"/>
-        <v>5.5788249592573336E-2</v>
+        <v>5.3402878242015228E-2</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
-        <v>5.578824959257334</v>
+        <v>5.340287824201523</v>
       </c>
       <c r="I25">
         <f t="shared" si="3"/>
-        <v>20.152549403915135</v>
+        <v>19.290874869584425</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -10450,21 +10675,27 @@
       <c r="B26">
         <v>0.7208099969006031</v>
       </c>
+      <c r="C26">
+        <v>0.74199673825976975</v>
+      </c>
+      <c r="D26">
+        <v>0.71856192261516894</v>
+      </c>
       <c r="E26">
         <f t="shared" si="0"/>
-        <v>0.7208099969006031</v>
+        <v>0.72712288592518048</v>
       </c>
       <c r="G26">
         <f t="shared" si="1"/>
-        <v>-4.011010157574546E-2</v>
+        <v>-3.3797212551168077E-2</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
-        <v>-4.011010157574546</v>
+        <v>-3.3797212551168077</v>
       </c>
       <c r="I26">
         <f t="shared" si="3"/>
-        <v>-5.2712632582660301</v>
+        <v>-4.4416243727617326</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -10474,21 +10705,27 @@
       <c r="B27">
         <v>0.29453861713409418</v>
       </c>
+      <c r="C27">
+        <v>0.29419887065887451</v>
+      </c>
+      <c r="D27">
+        <v>0.29453861713409418</v>
+      </c>
       <c r="E27">
         <f t="shared" si="0"/>
-        <v>0.29453861713409418</v>
+        <v>0.294425368309021</v>
       </c>
       <c r="G27">
         <f t="shared" si="1"/>
-        <v>1.2660741806030218E-2</v>
+        <v>1.2547492980957031E-2</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
-        <v>1.2660741806030218</v>
+        <v>1.2547492980957031</v>
       </c>
       <c r="I27">
         <f t="shared" si="3"/>
-        <v>4.4915699010768391</v>
+        <v>4.4513933441401221</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -10498,21 +10735,27 @@
       <c r="B28">
         <v>0.2101947218179703</v>
       </c>
+      <c r="C28">
+        <v>0.20935136079788211</v>
+      </c>
+      <c r="D28">
+        <v>0.2101947218179703</v>
+      </c>
       <c r="E28">
         <f t="shared" si="0"/>
-        <v>0.2101947218179703</v>
+        <v>0.20991360147794091</v>
       </c>
       <c r="G28">
         <f t="shared" si="1"/>
-        <v>6.2404026587804529E-3</v>
+        <v>5.9592823187510635E-3</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
-        <v>0.62404026587804529</v>
+        <v>0.59592823187510635</v>
       </c>
       <c r="I28">
         <f t="shared" si="3"/>
-        <v>3.0597060579578663</v>
+        <v>2.9218711049211668</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -10522,21 +10765,27 @@
       <c r="B29">
         <v>0.38173642754554749</v>
       </c>
+      <c r="C29">
+        <v>0.38190034031867981</v>
+      </c>
+      <c r="D29">
+        <v>0.38173642754554749</v>
+      </c>
       <c r="E29">
         <f t="shared" si="0"/>
-        <v>0.38173642754554749</v>
+        <v>0.38179106513659161</v>
       </c>
       <c r="G29">
         <f t="shared" si="1"/>
-        <v>1.947153608004254E-2</v>
+        <v>1.9526173671086666E-2</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
-        <v>1.947153608004254</v>
+        <v>1.9526173671086666</v>
       </c>
       <c r="I29">
         <f t="shared" si="3"/>
-        <v>5.3749442849050224</v>
+        <v>5.3900265057691792</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -10546,6 +10795,12 @@
       <c r="B30">
         <v>0.49640804597701149</v>
       </c>
+      <c r="C30">
+        <v>0.49640804597701149</v>
+      </c>
+      <c r="D30">
+        <v>0.49640804597701149</v>
+      </c>
       <c r="E30">
         <f t="shared" si="0"/>
         <v>0.49640804597701149</v>
@@ -10570,6 +10825,12 @@
       <c r="B31">
         <v>0.65517241379310343</v>
       </c>
+      <c r="C31">
+        <v>0.65517241379310343</v>
+      </c>
+      <c r="D31">
+        <v>0.65517241379310343</v>
+      </c>
       <c r="E31">
         <f t="shared" si="0"/>
         <v>0.65517241379310343</v>
@@ -10594,21 +10855,27 @@
       <c r="B32">
         <v>16.957900456313428</v>
       </c>
+      <c r="C32">
+        <v>14.593507018582571</v>
+      </c>
+      <c r="D32">
+        <v>14.76547417558473</v>
+      </c>
       <c r="E32">
         <f t="shared" si="0"/>
-        <v>16.957900456313428</v>
+        <v>15.438960550160244</v>
       </c>
       <c r="G32">
         <f t="shared" si="1"/>
-        <v>0.5995589549514051</v>
+        <v>-0.91938095120177898</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
-        <v>59.95589549514051</v>
+        <v>-91.938095120177906</v>
       </c>
       <c r="I32">
         <f t="shared" si="3"/>
-        <v>3.6651573443523282</v>
+        <v>-5.6202577206572544</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -10618,21 +10885,27 @@
       <c r="B33">
         <v>3361.7931034482758</v>
       </c>
+      <c r="C33">
+        <v>3380.5086206896549</v>
+      </c>
+      <c r="D33">
+        <v>3382.5775862068972</v>
+      </c>
       <c r="E33">
         <f t="shared" si="0"/>
-        <v>3361.7931034482758</v>
+        <v>3374.9597701149428</v>
       </c>
       <c r="G33">
         <f t="shared" si="1"/>
-        <v>210.92528735632231</v>
+        <v>224.09195402298928</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
-        <v>21092.52873563223</v>
+        <v>22409.19540229893</v>
       </c>
       <c r="I33">
         <f t="shared" si="3"/>
-        <v>6.6941966362122614</v>
+        <v>7.1120709310151993</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -10642,21 +10915,27 @@
       <c r="B34">
         <v>290.82758620689663</v>
       </c>
+      <c r="C34">
+        <v>294.61206896551732</v>
+      </c>
+      <c r="D34">
+        <v>293.25862068965517</v>
+      </c>
       <c r="E34">
         <f t="shared" si="0"/>
-        <v>290.82758620689663</v>
+        <v>292.89942528735634</v>
       </c>
       <c r="G34">
         <f t="shared" si="1"/>
-        <v>30.103448275862149</v>
+        <v>32.17528735632186</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
-        <v>3010.3448275862147</v>
+        <v>3217.528735632186</v>
       </c>
       <c r="I34">
         <f t="shared" si="3"/>
-        <v>11.546091786800719</v>
+        <v>12.340739761054543</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -10666,21 +10945,27 @@
       <c r="B35">
         <v>3652.620689655173</v>
       </c>
+      <c r="C35">
+        <v>3675.120689655173</v>
+      </c>
+      <c r="D35">
+        <v>3675.8362068965521</v>
+      </c>
       <c r="E35">
         <f t="shared" si="0"/>
-        <v>3652.620689655173</v>
+        <v>3667.8591954022995</v>
       </c>
       <c r="G35">
         <f t="shared" si="1"/>
-        <v>241.02873563218463</v>
+        <v>256.26724137931114</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
-        <v>24102.873563218462</v>
+        <v>25626.724137931116</v>
       </c>
       <c r="I35">
         <f t="shared" si="3"/>
-        <v>7.0649930847667992</v>
+        <v>7.511661559557786</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -10690,17 +10975,23 @@
       <c r="B36">
         <v>14503.793103448281</v>
       </c>
+      <c r="C36">
+        <v>14496.724137931031</v>
+      </c>
+      <c r="D36">
+        <v>14502.9224137931</v>
+      </c>
       <c r="E36">
         <f t="shared" si="0"/>
-        <v>14503.793103448281</v>
+        <v>14501.146551724138</v>
       </c>
       <c r="G36">
         <f t="shared" si="1"/>
-        <v>14503.793103448281</v>
+        <v>14501.146551724138</v>
       </c>
       <c r="H36">
         <f t="shared" si="2"/>
-        <v>1450379.3103448281</v>
+        <v>1450114.6551724137</v>
       </c>
       <c r="I36" t="e">
         <f t="shared" si="3"/>
@@ -10742,21 +11033,27 @@
       <c r="B40">
         <v>0.76993333772462869</v>
       </c>
+      <c r="C40">
+        <v>0.76577832767868992</v>
+      </c>
+      <c r="D40">
+        <v>0.77902954768266508</v>
+      </c>
       <c r="E40">
         <f>AVERAGE(B40:D40)</f>
-        <v>0.76993333772462869</v>
+        <v>0.7715804043619946</v>
       </c>
       <c r="G40">
         <f>E40-E3</f>
-        <v>-4.1835690864399422E-2</v>
+        <v>-4.0188624227033509E-2</v>
       </c>
       <c r="H40">
         <f>G40*100</f>
-        <v>-4.1835690864399417</v>
+        <v>-4.0188624227033509</v>
       </c>
       <c r="I40">
         <f>G40/E3*100</f>
-        <v>-5.1536446194696408</v>
+        <v>-4.9507461866199973</v>
       </c>
       <c r="J40" t="s">
         <v>26</v>
@@ -10769,21 +11066,27 @@
       <c r="B41">
         <v>0.7068504594820384</v>
       </c>
+      <c r="C41">
+        <v>0.70357142857142874</v>
+      </c>
+      <c r="D41">
+        <v>0.70375615763546795</v>
+      </c>
       <c r="E41">
         <f t="shared" ref="E41:E55" si="4">AVERAGE(B41:D41)</f>
-        <v>0.7068504594820384</v>
+        <v>0.70472601522964506</v>
       </c>
       <c r="G41">
         <f t="shared" ref="G41:G55" si="5">E41-E4</f>
-        <v>2.7806945524731397E-2</v>
+        <v>2.5682501272338065E-2</v>
       </c>
       <c r="H41">
         <f t="shared" ref="H41:H55" si="6">G41*100</f>
-        <v>2.7806945524731397</v>
+        <v>2.5682501272338065</v>
       </c>
       <c r="I41">
         <f t="shared" ref="I41:I55" si="7">G41/E4*100</f>
-        <v>4.0950167335638055</v>
+        <v>3.7821583955152511</v>
       </c>
       <c r="J41" t="s">
         <v>22</v>
@@ -10796,21 +11099,27 @@
       <c r="B42">
         <v>0.72522946857010362</v>
       </c>
+      <c r="C42">
+        <v>0.73678160916557645</v>
+      </c>
+      <c r="D42">
+        <v>0.73714080456775022</v>
+      </c>
       <c r="E42">
         <f t="shared" si="4"/>
-        <v>0.72522946857010362</v>
+        <v>0.7330506274344768</v>
       </c>
       <c r="G42">
         <f t="shared" si="5"/>
-        <v>7.4958076517650074E-2</v>
+        <v>8.2779235382023253E-2</v>
       </c>
       <c r="H42">
         <f t="shared" si="6"/>
-        <v>7.4958076517650074</v>
+        <v>8.2779235382023248</v>
       </c>
       <c r="I42">
         <f t="shared" si="7"/>
-        <v>11.527198864009637</v>
+        <v>12.729951892969934</v>
       </c>
       <c r="J42" t="s">
         <v>22</v>
@@ -10823,21 +11132,27 @@
       <c r="B43">
         <v>0.78722659826775332</v>
       </c>
+      <c r="C43">
+        <v>0.78727786122879417</v>
+      </c>
+      <c r="D43">
+        <v>0.78608559510084985</v>
+      </c>
       <c r="E43">
         <f t="shared" si="4"/>
-        <v>0.78722659826775332</v>
+        <v>0.78686335153246578</v>
       </c>
       <c r="G43">
         <f t="shared" si="5"/>
-        <v>3.2563161376112371E-3</v>
+        <v>2.8930694023237002E-3</v>
       </c>
       <c r="H43">
         <f t="shared" si="6"/>
-        <v>0.32563161376112371</v>
+        <v>0.28930694023237002</v>
       </c>
       <c r="I43">
         <f t="shared" si="7"/>
-        <v>0.41536219061307172</v>
+        <v>0.369027942546863</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -10847,21 +11162,27 @@
       <c r="B44">
         <v>0.27794117642294758</v>
       </c>
+      <c r="C44">
+        <v>0.27489079075862038</v>
+      </c>
+      <c r="D44">
+        <v>0.29159289196078908</v>
+      </c>
       <c r="E44">
         <f t="shared" si="4"/>
-        <v>0.27794117642294758</v>
+        <v>0.28147495304745235</v>
       </c>
       <c r="G44">
         <f t="shared" si="5"/>
-        <v>1.1114390313345934E-3</v>
+        <v>4.6452156558393631E-3</v>
       </c>
       <c r="H44">
         <f t="shared" si="6"/>
-        <v>0.11114390313345934</v>
+        <v>0.46452156558393631</v>
       </c>
       <c r="I44">
         <f t="shared" si="7"/>
-        <v>0.40148830895371368</v>
+        <v>1.6780045740779934</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -10871,21 +11192,27 @@
       <c r="B45">
         <v>0.70655532221611339</v>
       </c>
+      <c r="C45">
+        <v>0.71173713146123263</v>
+      </c>
+      <c r="D45">
+        <v>0.70874219736350841</v>
+      </c>
       <c r="E45">
         <f t="shared" si="4"/>
-        <v>0.70655532221611339</v>
+        <v>0.7090115503469514</v>
       </c>
       <c r="G45">
         <f t="shared" si="5"/>
-        <v>-5.436477626023517E-2</v>
+        <v>-5.1908548129397158E-2</v>
       </c>
       <c r="H45">
         <f t="shared" si="6"/>
-        <v>-5.4364776260235175</v>
+        <v>-5.1908548129397154</v>
       </c>
       <c r="I45">
         <f t="shared" si="7"/>
-        <v>-7.1446103696162222</v>
+        <v>-6.8218132538932554</v>
       </c>
       <c r="J45" t="s">
         <v>26</v>
@@ -10898,21 +11225,27 @@
       <c r="B46">
         <v>0.28015336394309998</v>
       </c>
+      <c r="C46">
+        <v>0.28015336394309998</v>
+      </c>
+      <c r="D46">
+        <v>0.27890640497207642</v>
+      </c>
       <c r="E46">
         <f t="shared" si="4"/>
-        <v>0.28015336394309998</v>
+        <v>0.27973771095275879</v>
       </c>
       <c r="G46">
         <f t="shared" si="5"/>
-        <v>-1.7245113849639893E-3</v>
+        <v>-2.1401643753051758E-3</v>
       </c>
       <c r="H46">
         <f t="shared" si="6"/>
-        <v>-0.17245113849639893</v>
+        <v>-0.21401643753051758</v>
       </c>
       <c r="I46">
         <f t="shared" si="7"/>
-        <v>-0.61179380714322262</v>
+        <v>-0.75925234387918616</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -10922,21 +11255,27 @@
       <c r="B47">
         <v>0.20270580053329471</v>
       </c>
+      <c r="C47">
+        <v>0.20270580053329471</v>
+      </c>
+      <c r="D47">
+        <v>0.20083476603031161</v>
+      </c>
       <c r="E47">
         <f t="shared" si="4"/>
-        <v>0.20270580053329471</v>
+        <v>0.20208212236563369</v>
       </c>
       <c r="G47">
         <f t="shared" si="5"/>
-        <v>-1.2485186258951453E-3</v>
+        <v>-1.8721967935561579E-3</v>
       </c>
       <c r="H47">
         <f t="shared" si="6"/>
-        <v>-0.12485186258951453</v>
+        <v>-0.18721967935561579</v>
       </c>
       <c r="I47">
         <f t="shared" si="7"/>
-        <v>-0.61215601171978862</v>
+        <v>-0.91794907863406228</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -10946,21 +11285,27 @@
       <c r="B48">
         <v>0.36114498972892761</v>
       </c>
+      <c r="C48">
+        <v>0.36114498972892761</v>
+      </c>
+      <c r="D48">
+        <v>0.36052832007408142</v>
+      </c>
       <c r="E48">
         <f t="shared" si="4"/>
-        <v>0.36114498972892761</v>
+        <v>0.3609394331773122</v>
       </c>
       <c r="G48">
         <f t="shared" si="5"/>
-        <v>-1.1199017365773334E-3</v>
+        <v>-1.325458288192749E-3</v>
       </c>
       <c r="H48">
         <f t="shared" si="6"/>
-        <v>-0.11199017365773334</v>
+        <v>-0.1325458288192749</v>
       </c>
       <c r="I48">
         <f t="shared" si="7"/>
-        <v>-0.30913890994153126</v>
+        <v>-0.36588096705445161</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -10970,6 +11315,12 @@
       <c r="B49">
         <v>0.41005747126436792</v>
       </c>
+      <c r="C49">
+        <v>0.41005747126436792</v>
+      </c>
+      <c r="D49">
+        <v>0.41005747126436792</v>
+      </c>
       <c r="E49">
         <f t="shared" si="4"/>
         <v>0.41005747126436792</v>
@@ -10997,6 +11348,12 @@
       <c r="B50">
         <v>0.59482758620689657</v>
       </c>
+      <c r="C50">
+        <v>0.59482758620689657</v>
+      </c>
+      <c r="D50">
+        <v>0.59482758620689657</v>
+      </c>
       <c r="E50">
         <f t="shared" si="4"/>
         <v>0.59482758620689657</v>
@@ -11024,21 +11381,27 @@
       <c r="B51">
         <v>15.383776977144439</v>
       </c>
+      <c r="C51">
+        <v>16.153961255632598</v>
+      </c>
+      <c r="D51">
+        <v>14.66555479477192</v>
+      </c>
       <c r="E51">
         <f t="shared" si="4"/>
-        <v>15.383776977144439</v>
+        <v>15.401097675849654</v>
       </c>
       <c r="G51">
         <f t="shared" si="5"/>
-        <v>-0.97456452421758399</v>
+        <v>-0.95724382551236964</v>
       </c>
       <c r="H51">
         <f t="shared" si="6"/>
-        <v>-97.456452421758399</v>
+        <v>-95.724382551236971</v>
       </c>
       <c r="I51">
         <f t="shared" si="7"/>
-        <v>-5.9575998223074151</v>
+        <v>-5.8517168469228249</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
@@ -11048,21 +11411,27 @@
       <c r="B52">
         <v>3389.974137931034</v>
       </c>
+      <c r="C52">
+        <v>3389.974137931034</v>
+      </c>
+      <c r="D52">
+        <v>3388.2327586206902</v>
+      </c>
       <c r="E52">
         <f t="shared" si="4"/>
-        <v>3389.974137931034</v>
+        <v>3389.3936781609191</v>
       </c>
       <c r="G52">
         <f t="shared" si="5"/>
-        <v>239.10632183908046</v>
+        <v>238.52586206896558</v>
       </c>
       <c r="H52">
         <f t="shared" si="6"/>
-        <v>23910.632183908048</v>
+        <v>23852.586206896558</v>
       </c>
       <c r="I52">
         <f t="shared" si="7"/>
-        <v>7.5885862497286833</v>
+        <v>7.5701640307085647</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
@@ -11072,21 +11441,27 @@
       <c r="B53">
         <v>275.91379310344831</v>
       </c>
+      <c r="C53">
+        <v>275.91379310344831</v>
+      </c>
+      <c r="D53">
+        <v>276.65517241379308</v>
+      </c>
       <c r="E53">
         <f t="shared" si="4"/>
-        <v>275.91379310344831</v>
+        <v>276.16091954022994</v>
       </c>
       <c r="G53">
         <f t="shared" si="5"/>
-        <v>15.189655172413836</v>
+        <v>15.436781609195464</v>
       </c>
       <c r="H53">
         <f t="shared" si="6"/>
-        <v>1518.9655172413836</v>
+        <v>1543.6781609195464</v>
       </c>
       <c r="I53">
         <f t="shared" si="7"/>
-        <v>5.8259489485517957</v>
+        <v>5.9207335890314567</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
@@ -11096,21 +11471,27 @@
       <c r="B54">
         <v>3665.8879310344828</v>
       </c>
+      <c r="C54">
+        <v>3665.8879310344828</v>
+      </c>
+      <c r="D54">
+        <v>3664.8879310344828</v>
+      </c>
       <c r="E54">
         <f t="shared" si="4"/>
-        <v>3665.8879310344828</v>
+        <v>3665.5545977011498</v>
       </c>
       <c r="G54">
         <f t="shared" si="5"/>
-        <v>254.29597701149441</v>
+        <v>253.96264367816138</v>
       </c>
       <c r="H54">
         <f t="shared" si="6"/>
-        <v>25429.59770114944</v>
+        <v>25396.26436781614</v>
       </c>
       <c r="I54">
         <f t="shared" si="7"/>
-        <v>7.4538801954795817</v>
+        <v>7.4441095858103932</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
@@ -11120,17 +11501,23 @@
       <c r="B55">
         <v>12648.586206896551</v>
       </c>
+      <c r="C55">
+        <v>12648.1724137931</v>
+      </c>
+      <c r="D55">
+        <v>12651.11206896552</v>
+      </c>
       <c r="E55">
         <f t="shared" si="4"/>
-        <v>12648.586206896551</v>
+        <v>12649.290229885059</v>
       </c>
       <c r="G55">
         <f t="shared" si="5"/>
-        <v>12648.586206896551</v>
+        <v>12649.290229885059</v>
       </c>
       <c r="H55">
         <f t="shared" si="6"/>
-        <v>1264858.6206896552</v>
+        <v>1264929.0229885059</v>
       </c>
       <c r="I55" t="e">
         <f t="shared" si="7"/>
@@ -13776,7 +14163,7 @@
         <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="H2" t="s">
         <v>20</v>
@@ -14856,21 +15243,27 @@
       <c r="B21">
         <v>0.78010525375598061</v>
       </c>
+      <c r="C21">
+        <v>0.77389086260835749</v>
+      </c>
+      <c r="D21">
+        <v>0.76431684118725984</v>
+      </c>
       <c r="E21">
         <f>AVERAGE(B21:D21)</f>
-        <v>0.78010525375598061</v>
+        <v>0.77277098585053261</v>
       </c>
       <c r="G21">
         <f>E21-E3</f>
-        <v>-3.1663774833047498E-2</v>
+        <v>-3.8998042738495498E-2</v>
       </c>
       <c r="H21">
         <f>G21*100</f>
-        <v>-3.1663774833047498</v>
+        <v>-3.8998042738495498</v>
       </c>
       <c r="I21">
         <f>G21/E3*100</f>
-        <v>-3.9005891722776997</v>
+        <v>-4.8040811320776466</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -14880,21 +15273,27 @@
       <c r="B22">
         <v>0.66709770114942524</v>
       </c>
+      <c r="C22">
+        <v>0.68545258620689653</v>
+      </c>
+      <c r="D22">
+        <v>0.67614942528735633</v>
+      </c>
       <c r="E22">
         <f t="shared" ref="E22:E35" si="0">AVERAGE(B22:D22)</f>
-        <v>0.66709770114942524</v>
+        <v>0.67623323754789266</v>
       </c>
       <c r="G22">
         <f t="shared" ref="G22:G35" si="1">E22-E4</f>
-        <v>-1.1945812807881762E-2</v>
+        <v>-2.8102764094143362E-3</v>
       </c>
       <c r="H22">
         <f t="shared" ref="H22:H35" si="2">G22*100</f>
-        <v>-1.1945812807881762</v>
+        <v>-0.28102764094143362</v>
       </c>
       <c r="I22">
         <f t="shared" ref="I22:I35" si="3">G22/E4*100</f>
-        <v>-1.7592116797146555</v>
+        <v>-0.41385807413676656</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -14904,21 +15303,27 @@
       <c r="B23">
         <v>0.64701867813004521</v>
       </c>
+      <c r="C23">
+        <v>0.62733477008614202</v>
+      </c>
+      <c r="D23">
+        <v>0.6258860152955914</v>
+      </c>
       <c r="E23">
         <f t="shared" si="0"/>
-        <v>0.64701867813004521</v>
+        <v>0.63341315450392621</v>
       </c>
       <c r="G23">
         <f t="shared" si="1"/>
-        <v>-3.2527139224083346E-3</v>
+        <v>-1.6858237548527333E-2</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
-        <v>-0.32527139224083346</v>
+        <v>-1.6858237548527333</v>
       </c>
       <c r="I23">
         <f t="shared" si="3"/>
-        <v>-0.50020867627926613</v>
+        <v>-2.59249257380332</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -14928,21 +15333,27 @@
       <c r="B24">
         <v>0.77736996807890157</v>
       </c>
+      <c r="C24">
+        <v>0.77713869036916794</v>
+      </c>
+      <c r="D24">
+        <v>0.77828712535580014</v>
+      </c>
       <c r="E24">
         <f t="shared" si="0"/>
-        <v>0.77736996807890157</v>
+        <v>0.77759859460128988</v>
       </c>
       <c r="G24">
         <f t="shared" si="1"/>
-        <v>-6.6003140512405079E-3</v>
+        <v>-6.371687528852199E-3</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
-        <v>-0.66003140512405079</v>
+        <v>-0.6371687528852199</v>
       </c>
       <c r="I24">
         <f t="shared" si="3"/>
-        <v>-0.84190870517523386</v>
+        <v>-0.81274605352891094</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -14952,21 +15363,27 @@
       <c r="B25">
         <v>0.27990844108872298</v>
       </c>
+      <c r="C25">
+        <v>0.29509227238341967</v>
+      </c>
+      <c r="D25">
+        <v>0.28152644851893482</v>
+      </c>
       <c r="E25">
         <f t="shared" si="0"/>
-        <v>0.27990844108872298</v>
+        <v>0.28550905399702581</v>
       </c>
       <c r="G25">
         <f t="shared" si="1"/>
-        <v>3.0787036971099968E-3</v>
+        <v>8.6793166054128235E-3</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
-        <v>0.30787036971099968</v>
+        <v>0.86793166054128235</v>
       </c>
       <c r="I25">
         <f t="shared" si="3"/>
-        <v>1.1121289663887357</v>
+        <v>3.1352544301029193</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -14976,21 +15393,27 @@
       <c r="B26">
         <v>0.69277850660982321</v>
       </c>
+      <c r="C26">
+        <v>0.68286122554372364</v>
+      </c>
+      <c r="D26">
+        <v>0.6956917532452741</v>
+      </c>
       <c r="E26">
         <f t="shared" si="0"/>
-        <v>0.69277850660982321</v>
+        <v>0.69044382846627361</v>
       </c>
       <c r="G26">
         <f t="shared" si="1"/>
-        <v>-6.8141591866525353E-2</v>
+        <v>-7.0476270010074948E-2</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
-        <v>-6.8141591866525353</v>
+        <v>-7.0476270010074948</v>
       </c>
       <c r="I26">
         <f t="shared" si="3"/>
-        <v>-8.9551573158562565</v>
+        <v>-9.261980351313527</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -15000,21 +15423,27 @@
       <c r="B27">
         <v>0.28047475218772888</v>
       </c>
+      <c r="C27">
+        <v>0.27995514869689941</v>
+      </c>
+      <c r="D27">
+        <v>0.27759167551994318</v>
+      </c>
       <c r="E27">
         <f t="shared" si="0"/>
-        <v>0.28047475218772888</v>
+        <v>0.27934052546819049</v>
       </c>
       <c r="G27">
         <f t="shared" si="1"/>
-        <v>-1.403123140335083E-3</v>
+        <v>-2.5373498598734723E-3</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
-        <v>-0.1403123140335083</v>
+        <v>-0.25373498598734723</v>
       </c>
       <c r="I27">
         <f t="shared" si="3"/>
-        <v>-0.49777696766802154</v>
+        <v>-0.90015928242696375</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -15024,21 +15453,27 @@
       <c r="B28">
         <v>0.2093124836683273</v>
       </c>
+      <c r="C28">
+        <v>0.208344966173172</v>
+      </c>
+      <c r="D28">
+        <v>0.20594584941864011</v>
+      </c>
       <c r="E28">
         <f t="shared" si="0"/>
-        <v>0.2093124836683273</v>
+        <v>0.20786776642004648</v>
       </c>
       <c r="G28">
         <f t="shared" si="1"/>
-        <v>5.358164509137453E-3</v>
+        <v>3.9134472608566284E-3</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
-        <v>0.5358164509137453</v>
+        <v>0.39134472608566284</v>
       </c>
       <c r="I28">
         <f t="shared" si="3"/>
-        <v>2.627139513998384</v>
+        <v>1.9187861659365573</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -15048,21 +15483,27 @@
       <c r="B29">
         <v>0.35389664769172668</v>
       </c>
+      <c r="C29">
+        <v>0.35387969017028809</v>
+      </c>
+      <c r="D29">
+        <v>0.3515298068523407</v>
+      </c>
       <c r="E29">
         <f t="shared" si="0"/>
-        <v>0.35389664769172668</v>
+        <v>0.35310204823811847</v>
       </c>
       <c r="G29">
         <f t="shared" si="1"/>
-        <v>-8.3682437737782611E-3</v>
+        <v>-9.1628432273864746E-3</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
-        <v>-0.83682437737782611</v>
+        <v>-0.91628432273864746</v>
       </c>
       <c r="I29">
         <f t="shared" si="3"/>
-        <v>-2.3099792364436422</v>
+        <v>-2.5293213455819981</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -15072,21 +15513,27 @@
       <c r="B30">
         <v>0.35632183908045978</v>
       </c>
+      <c r="C30">
+        <v>0.35632183908045978</v>
+      </c>
+      <c r="D30">
+        <v>0.35775862068965519</v>
+      </c>
       <c r="E30">
         <f t="shared" si="0"/>
-        <v>0.35632183908045978</v>
+        <v>0.35680076628352492</v>
       </c>
       <c r="G30">
         <f t="shared" si="1"/>
-        <v>-2.8208812260536342E-2</v>
+        <v>-2.7729885057471204E-2</v>
       </c>
       <c r="H30">
         <f t="shared" si="2"/>
-        <v>-2.8208812260536344</v>
+        <v>-2.7729885057471204</v>
       </c>
       <c r="I30">
         <f t="shared" si="3"/>
-        <v>-7.335907335907323</v>
+        <v>-7.2113588242620343</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -15096,6 +15543,12 @@
       <c r="B31">
         <v>0.53448275862068961</v>
       </c>
+      <c r="C31">
+        <v>0.53448275862068961</v>
+      </c>
+      <c r="D31">
+        <v>0.53448275862068961</v>
+      </c>
       <c r="E31">
         <f t="shared" si="0"/>
         <v>0.53448275862068961</v>
@@ -15120,21 +15573,27 @@
       <c r="B32">
         <v>16.306659532004389</v>
       </c>
+      <c r="C32">
+        <v>16.24340450352636</v>
+      </c>
+      <c r="D32">
+        <v>14.72616429781092</v>
+      </c>
       <c r="E32">
         <f t="shared" si="0"/>
-        <v>16.306659532004389</v>
+        <v>15.758742777780556</v>
       </c>
       <c r="G32">
         <f t="shared" si="1"/>
-        <v>-5.1681969357634472E-2</v>
+        <v>-0.59959872358146704</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
-        <v>-5.1681969357634472</v>
+        <v>-59.959872358146704</v>
       </c>
       <c r="I32">
         <f t="shared" si="3"/>
-        <v>-0.31593648630780413</v>
+        <v>-3.6654004535334064</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -15144,21 +15603,27 @@
       <c r="B33">
         <v>3536.094827586207</v>
       </c>
+      <c r="C33">
+        <v>3536.3965517241381</v>
+      </c>
+      <c r="D33">
+        <v>3536.3189655172409</v>
+      </c>
       <c r="E33">
         <f t="shared" si="0"/>
-        <v>3536.094827586207</v>
+        <v>3536.2701149425288</v>
       </c>
       <c r="G33">
         <f t="shared" si="1"/>
-        <v>385.22701149425347</v>
+        <v>385.40229885057533</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
-        <v>38522.701149425346</v>
+        <v>38540.229885057532</v>
       </c>
       <c r="I33">
         <f t="shared" si="3"/>
-        <v>12.226060691179791</v>
+        <v>12.231623836527451</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -15168,21 +15633,27 @@
       <c r="B34">
         <v>256.75</v>
       </c>
+      <c r="C34">
+        <v>257.15517241379308</v>
+      </c>
+      <c r="D34">
+        <v>257.00862068965517</v>
+      </c>
       <c r="E34">
         <f t="shared" si="0"/>
-        <v>256.75</v>
+        <v>256.97126436781605</v>
       </c>
       <c r="G34">
         <f t="shared" si="1"/>
-        <v>-3.9741379310344769</v>
+        <v>-3.7528735632184294</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
-        <v>-397.41379310344769</v>
+        <v>-375.28735632184294</v>
       </c>
       <c r="I34">
         <f t="shared" si="3"/>
-        <v>-1.5242692765507186</v>
+        <v>-1.4394039589119754</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -15192,21 +15663,27 @@
       <c r="B35">
         <v>3792.844827586207</v>
       </c>
+      <c r="C35">
+        <v>3793.5517241379312</v>
+      </c>
+      <c r="D35">
+        <v>3793.3275862068972</v>
+      </c>
       <c r="E35">
         <f t="shared" si="0"/>
-        <v>3792.844827586207</v>
+        <v>3793.2413793103447</v>
       </c>
       <c r="G35">
         <f t="shared" si="1"/>
-        <v>381.2528735632186</v>
+        <v>381.64942528735628</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
-        <v>38125.28735632186</v>
+        <v>38164.942528735628</v>
       </c>
       <c r="I35">
         <f t="shared" si="3"/>
-        <v>11.175219038538323</v>
+        <v>11.186842694868913</v>
       </c>
     </row>
   </sheetData>

</xml_diff>